<commit_message>
Update some data in database_inventory
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE48087E-5742-48A3-A5E8-BCCACA78E40B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF8BC072-1C99-4149-884D-778F18DA6CE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="71">
   <si>
     <t>Database No.</t>
   </si>
@@ -216,12 +216,6 @@
     <t xml:space="preserve">Participant </t>
   </si>
   <si>
-    <t>Weight(KG)</t>
-  </si>
-  <si>
-    <t>Height(CM)</t>
-  </si>
-  <si>
     <t>Weight</t>
   </si>
   <si>
@@ -241,6 +235,24 @@
   </si>
   <si>
     <t>Grouvel</t>
+  </si>
+  <si>
+    <t>Height (cm)</t>
+  </si>
+  <si>
+    <t>Calib pose</t>
+  </si>
+  <si>
+    <t>Walk trials (files)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usable Walk trials </t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Duration per trials</t>
   </si>
 </sst>
 </file>
@@ -652,7 +664,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -667,7 +679,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D5">
         <v>2023</v>
@@ -798,15 +810,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
     <col min="4" max="4" width="14.109375" customWidth="1"/>
     <col min="5" max="5" width="12.21875" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" customWidth="1"/>
+    <col min="8" max="8" width="14.6640625" customWidth="1"/>
+    <col min="9" max="9" width="16.33203125" customWidth="1"/>
+    <col min="10" max="10" width="16.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -820,10 +836,22 @@
         <v>53</v>
       </c>
       <c r="E1" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>62</v>
+      </c>
+      <c r="G1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <f t="shared" ref="A2:A31" si="0">ROW(A1)</f>
         <v>1</v>
@@ -841,7 +869,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <f t="shared" si="0"/>
         <v>2</v>
@@ -859,7 +887,7 @@
         <v>1730</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <f t="shared" si="0"/>
         <v>3</v>
@@ -877,7 +905,7 @@
         <v>1700</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -895,7 +923,7 @@
         <v>1870</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -913,7 +941,7 @@
         <v>1640</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -931,7 +959,7 @@
         <v>1830</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -949,7 +977,7 @@
         <v>1840</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -967,7 +995,7 @@
         <v>1700</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -985,7 +1013,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1003,7 +1031,7 @@
         <v>1740</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1021,7 +1049,7 @@
         <v>1630</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1039,7 +1067,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1057,7 +1085,7 @@
         <v>1760</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1075,7 +1103,7 @@
         <v>1680</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1371,15 +1399,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.77734375" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="5" max="5" width="16.44140625" customWidth="1"/>
+    <col min="4" max="4" width="10.77734375" customWidth="1"/>
+    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" customWidth="1"/>
+    <col min="7" max="7" width="9.88671875" customWidth="1"/>
+    <col min="8" max="8" width="14.109375" customWidth="1"/>
+    <col min="9" max="9" width="16.88671875" customWidth="1"/>
+    <col min="10" max="10" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1390,13 +1423,25 @@
         <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+      <c r="G1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1412,8 +1457,14 @@
       <c r="E2">
         <v>175</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1429,8 +1480,14 @@
       <c r="E3">
         <v>172</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1446,8 +1503,14 @@
       <c r="E4">
         <v>178</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1463,8 +1526,14 @@
       <c r="E5">
         <v>170</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1480,8 +1549,14 @@
       <c r="E6">
         <v>171</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G6">
+        <v>1</v>
+      </c>
+      <c r="H6">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1497,8 +1572,14 @@
       <c r="E7">
         <v>168</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1514,8 +1595,14 @@
       <c r="E8">
         <v>176</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1531,8 +1618,14 @@
       <c r="E9">
         <v>181</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1548,8 +1641,14 @@
       <c r="E10">
         <v>183</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G10">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1565,8 +1664,14 @@
       <c r="E11">
         <v>182</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1582,8 +1687,14 @@
       <c r="E12">
         <v>175</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1599,8 +1710,14 @@
       <c r="E13">
         <v>177</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1615,6 +1732,12 @@
       </c>
       <c r="E14">
         <v>170</v>
+      </c>
+      <c r="G14">
+        <v>1</v>
+      </c>
+      <c r="H14">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1625,10 +1748,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="16.44140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1639,10 +1766,132 @@
         <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E1" t="s">
         <v>54</v>
+      </c>
+      <c r="G1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="G4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1653,14 +1902,18 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="14.6640625" customWidth="1"/>
     <col min="4" max="4" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="9.6640625" customWidth="1"/>
+    <col min="8" max="8" width="14.77734375" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="17.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1671,18 +1924,30 @@
         <v>52</v>
       </c>
       <c r="D1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+        <v>60</v>
+      </c>
+      <c r="G1" t="s">
+        <v>66</v>
+      </c>
+      <c r="H1" t="s">
+        <v>67</v>
+      </c>
+      <c r="I1" t="s">
+        <v>68</v>
+      </c>
+      <c r="J1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C2" t="s">
         <v>55</v>
@@ -1694,12 +1959,12 @@
         <v>1.68</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C3" t="s">
         <v>56</v>
@@ -1711,12 +1976,12 @@
         <v>1.7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C4" t="s">
         <v>55</v>
@@ -1728,12 +1993,12 @@
         <v>1.59</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C5" t="s">
         <v>56</v>
@@ -1745,12 +2010,12 @@
         <v>1.82</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C6" t="s">
         <v>56</v>
@@ -1762,12 +2027,12 @@
         <v>1.95</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C7" t="s">
         <v>55</v>
@@ -1779,12 +2044,12 @@
         <v>1.53</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Update database_inventory, wrong trials
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2D0001A-200C-4C9A-BE47-B918FFBC54A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A88D27DC-FC7F-430F-B51B-66DAE71764CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="77">
   <si>
     <t>Database No.</t>
   </si>
@@ -237,24 +237,15 @@
     <t>Weight (kg)</t>
   </si>
   <si>
-    <t>Height (mm)</t>
-  </si>
-  <si>
     <t>Calib pose</t>
   </si>
   <si>
     <t>Walk trials (files)</t>
   </si>
   <si>
-    <t>Duration per trials</t>
-  </si>
-  <si>
     <t xml:space="preserve">Participant </t>
   </si>
   <si>
-    <t>Height (cm)</t>
-  </si>
-  <si>
     <t>M</t>
   </si>
   <si>
@@ -270,9 +261,6 @@
     <t xml:space="preserve">Usable trials </t>
   </si>
   <si>
-    <t>Walk trials</t>
-  </si>
-  <si>
     <t>Duration per trials (s)</t>
   </si>
   <si>
@@ -280,9 +268,6 @@
   </si>
   <si>
     <t>Height (m)</t>
-  </si>
-  <si>
-    <t>Participant</t>
   </si>
   <si>
     <t>1:3 (No ID)</t>
@@ -908,21 +893,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:K1"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" customWidth="1"/>
-    <col min="4" max="4" width="14.109375" customWidth="1"/>
-    <col min="5" max="5" width="12.21875" customWidth="1"/>
-    <col min="7" max="7" width="11.6640625" customWidth="1"/>
-    <col min="8" max="8" width="14.6640625" customWidth="1"/>
-    <col min="9" max="9" width="16.33203125" customWidth="1"/>
-    <col min="10" max="10" width="16.77734375" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" customWidth="1"/>
+    <col min="4" max="5" width="8.77734375" customWidth="1"/>
+    <col min="7" max="10" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>60</v>
@@ -934,19 +915,22 @@
         <v>62</v>
       </c>
       <c r="E1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G1" t="s">
         <v>63</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s">
-        <v>74</v>
-      </c>
       <c r="I1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J1" t="s">
-        <v>66</v>
+        <v>71</v>
+      </c>
+      <c r="K1" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -957,22 +941,16 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.77734375" customWidth="1"/>
-    <col min="4" max="4" width="10.77734375" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" customWidth="1"/>
-    <col min="7" max="7" width="9.88671875" customWidth="1"/>
-    <col min="8" max="8" width="14.109375" customWidth="1"/>
-    <col min="9" max="9" width="16.88671875" customWidth="1"/>
-    <col min="10" max="10" width="16.6640625" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" customWidth="1"/>
+    <col min="4" max="10" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>60</v>
@@ -984,22 +962,25 @@
         <v>62</v>
       </c>
       <c r="E1" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="G1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s">
-        <v>65</v>
-      </c>
       <c r="I1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+      <c r="K1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1007,7 +988,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2">
         <v>74</v>
@@ -1021,8 +1002,11 @@
       <c r="H2">
         <v>21</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K2" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1030,7 +1014,7 @@
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D3">
         <v>72</v>
@@ -1044,8 +1028,11 @@
       <c r="H3">
         <v>23</v>
       </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1053,7 +1040,7 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D4">
         <v>80</v>
@@ -1067,8 +1054,11 @@
       <c r="H4">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="K4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1076,7 +1066,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D5">
         <v>60</v>
@@ -1091,7 +1081,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1099,7 +1089,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D6">
         <v>71</v>
@@ -1114,7 +1104,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1122,7 +1112,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D7">
         <v>65</v>
@@ -1137,7 +1127,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1145,7 +1135,7 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D8">
         <v>72</v>
@@ -1160,7 +1150,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1168,7 +1158,7 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D9">
         <v>85</v>
@@ -1183,7 +1173,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1191,7 +1181,7 @@
         <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D10">
         <v>76</v>
@@ -1206,7 +1196,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1214,7 +1204,7 @@
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D11">
         <v>80</v>
@@ -1229,7 +1219,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1237,7 +1227,7 @@
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D12">
         <v>75</v>
@@ -1252,7 +1242,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1260,7 +1250,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D13">
         <v>80</v>
@@ -1275,7 +1265,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1283,7 +1273,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D14">
         <v>58</v>
@@ -1314,7 +1304,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>60</v>
@@ -1326,22 +1316,22 @@
         <v>62</v>
       </c>
       <c r="E1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s">
-        <v>65</v>
-      </c>
       <c r="I1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1349,25 +1339,22 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G2">
         <v>0</v>
       </c>
       <c r="H2">
         <v>18</v>
-      </c>
-      <c r="K2" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -1375,25 +1362,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G3">
         <v>0</v>
       </c>
       <c r="H3">
         <v>16</v>
-      </c>
-      <c r="K3">
-        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -1401,25 +1385,22 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G4">
         <v>0</v>
       </c>
       <c r="H4">
         <v>12</v>
-      </c>
-      <c r="K4">
-        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
@@ -1427,16 +1408,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1450,16 +1431,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1473,16 +1454,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1496,16 +1477,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1519,16 +1500,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -1542,16 +1523,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1565,16 +1546,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1601,7 +1582,7 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B1" t="s">
         <v>60</v>
@@ -1613,22 +1594,22 @@
         <v>62</v>
       </c>
       <c r="E1" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="G1" t="s">
+        <v>63</v>
+      </c>
+      <c r="H1" t="s">
         <v>64</v>
       </c>
-      <c r="H1" t="s">
-        <v>65</v>
-      </c>
       <c r="I1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="K1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
@@ -1636,10 +1617,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C2" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D2">
         <v>69.86</v>
@@ -1651,7 +1632,7 @@
         <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
@@ -1659,10 +1640,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D3">
         <v>66.680000000000007</v>
@@ -1674,7 +1655,7 @@
         <v>4</v>
       </c>
       <c r="K3" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
@@ -1682,10 +1663,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D4">
         <v>53.07</v>
@@ -1702,10 +1683,10 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D5">
         <v>71.67</v>
@@ -1722,10 +1703,10 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D6">
         <v>90.7</v>
@@ -1742,10 +1723,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C7" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D7">
         <v>48.99</v>
@@ -1762,10 +1743,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D8">
         <v>63.96</v>

</xml_diff>

<commit_message>
Update inventory sheet with DB1 details.
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/TeamProject/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6966347-513D-4FED-BBDA-268D7F849F99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF009508-D356-0346-BFB3-6CF22E7AFCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="27420" windowHeight="17500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -29,12 +29,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="93">
   <si>
     <t>Database No.</t>
-  </si>
-  <si>
-    <t>Related Paper</t>
   </si>
   <si>
     <t>Authors</t>
@@ -292,12 +289,69 @@
   <si>
     <t>Self-selected spontaneous (C4) and fast (C5)</t>
   </si>
+  <si>
+    <t>A multimodal dataset of human gait at different walking speeds established on injury-free adult participants</t>
+  </si>
+  <si>
+    <t>Schreiber &amp; Moissenet</t>
+  </si>
+  <si>
+    <t>19-67</t>
+  </si>
+  <si>
+    <t>1.74 ± 0.09 m</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">71.0 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="EuclidSymbol"/>
+      </rPr>
+      <t xml:space="preserve">± </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="MinionPro"/>
+      </rPr>
+      <t xml:space="preserve">12.3 kg </t>
+    </r>
+  </si>
+  <si>
+    <t>5 trials each with 5 different speeds</t>
+  </si>
+  <si>
+    <t>Luxembourg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">52 reflective markers </t>
+  </si>
+  <si>
+    <t>https://figshare.com/articles/dataset/A_multimodal_dataset_of_human_gait_at_different_walking_speeds/7734767</t>
+  </si>
+  <si>
+    <t>W</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1-C5 variable trails </t>
+  </si>
+  <si>
+    <t>only C4 &amp; C5 (variable trials)</t>
+  </si>
+  <si>
+    <t>Duration per trials(s)</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -334,6 +388,36 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="MinionPro"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="EuclidSymbol"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -357,7 +441,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -367,6 +451,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -562,119 +656,164 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:R11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" customWidth="1"/>
-    <col min="2" max="2" width="17.77734375" customWidth="1"/>
-    <col min="4" max="4" width="14.33203125" customWidth="1"/>
-    <col min="5" max="5" width="33.77734375" customWidth="1"/>
-    <col min="6" max="6" width="36" customWidth="1"/>
-    <col min="7" max="7" width="23.6640625" customWidth="1"/>
-    <col min="8" max="8" width="13.44140625" customWidth="1"/>
-    <col min="10" max="10" width="9.77734375" customWidth="1"/>
-    <col min="11" max="11" width="12.6640625" customWidth="1"/>
-    <col min="12" max="12" width="14.33203125" customWidth="1"/>
-    <col min="13" max="13" width="12.6640625" customWidth="1"/>
-    <col min="14" max="14" width="20" customWidth="1"/>
-    <col min="15" max="15" width="28.44140625" customWidth="1"/>
-    <col min="16" max="16" width="24.44140625" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
-    <col min="18" max="18" width="13" customWidth="1"/>
-    <col min="19" max="19" width="29.77734375" customWidth="1"/>
+    <col min="1" max="1" width="11.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1640625" customWidth="1"/>
+    <col min="4" max="4" width="33.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36" customWidth="1"/>
+    <col min="6" max="6" width="23.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.5" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" customWidth="1"/>
+    <col min="12" max="12" width="12.6640625" customWidth="1"/>
+    <col min="13" max="13" width="20" customWidth="1"/>
+    <col min="14" max="14" width="28.5" customWidth="1"/>
+    <col min="15" max="15" width="24.5" customWidth="1"/>
+    <col min="16" max="16" width="20" customWidth="1"/>
+    <col min="17" max="17" width="40.83203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:18" s="6" customFormat="1" ht="17">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:18" ht="64">
       <c r="A2">
         <v>1</v>
       </c>
-      <c r="G2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2">
+        <v>2019</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G2">
+        <v>50</v>
+      </c>
+      <c r="H2">
+        <v>24</v>
+      </c>
+      <c r="I2">
+        <v>26</v>
+      </c>
+      <c r="J2" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2" t="s">
+        <v>84</v>
+      </c>
+      <c r="M2" t="s">
+        <v>86</v>
+      </c>
+      <c r="N2" t="s">
+        <v>85</v>
+      </c>
+      <c r="O2" t="s">
+        <v>87</v>
+      </c>
+      <c r="P2">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" ht="48">
       <c r="A3">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B3" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3">
+        <v>2025</v>
+      </c>
+      <c r="D3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D3">
-        <v>2025</v>
-      </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3">
+        <v>13</v>
+      </c>
+      <c r="H3" s="1">
+        <v>0</v>
+      </c>
+      <c r="I3" s="1">
+        <v>13</v>
+      </c>
+      <c r="J3" t="s">
         <v>20</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="H3">
-        <v>13</v>
-      </c>
-      <c r="I3" s="1">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1">
-        <v>13</v>
       </c>
       <c r="K3" t="s">
         <v>21</v>
@@ -682,87 +821,87 @@
       <c r="L3" t="s">
         <v>22</v>
       </c>
-      <c r="M3" t="s">
+      <c r="O3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="R3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="S3" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="4" spans="1:19" ht="46.8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:18" ht="51">
       <c r="A4">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="B4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4">
+        <v>2023</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D4">
-        <v>2023</v>
-      </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="G4" s="1">
+        <v>10</v>
+      </c>
+      <c r="H4" s="1">
+        <v>4</v>
+      </c>
+      <c r="I4" s="1">
+        <v>6</v>
+      </c>
+      <c r="J4" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="1">
-        <v>10</v>
-      </c>
-      <c r="I4" s="1">
-        <v>4</v>
-      </c>
-      <c r="J4" s="1">
-        <v>6</v>
-      </c>
-      <c r="K4" s="1" t="s">
+      <c r="K4" s="2" t="s">
         <v>28</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="M4" s="2" t="s">
+      <c r="O4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="R4" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="S4" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
+    </row>
+    <row r="5" spans="1:18" ht="48">
       <c r="A5">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="B5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5">
+        <v>2023</v>
+      </c>
+      <c r="D5" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D5">
-        <v>2023</v>
-      </c>
       <c r="E5" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="1">
+        <v>7</v>
+      </c>
+      <c r="H5" s="1">
+        <v>4</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3</v>
+      </c>
+      <c r="J5" t="s">
         <v>35</v>
-      </c>
-      <c r="H5" s="1">
-        <v>7</v>
-      </c>
-      <c r="I5" s="1">
-        <v>4</v>
-      </c>
-      <c r="J5" s="1">
-        <v>3</v>
       </c>
       <c r="K5" t="s">
         <v>36</v>
@@ -770,43 +909,41 @@
       <c r="L5" t="s">
         <v>37</v>
       </c>
-      <c r="M5" t="s">
+      <c r="O5" s="1">
+        <v>96</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="P5" s="1">
-        <v>96</v>
-      </c>
-      <c r="R5" t="s">
+      <c r="R5" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="S5" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:18">
+      <c r="D7" s="1"/>
       <c r="E7" s="1"/>
-      <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
       <c r="I7" s="1"/>
-      <c r="J7" s="1"/>
-      <c r="S7" s="1"/>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="R7" s="1"/>
+    </row>
+    <row r="8" spans="1:18">
+      <c r="D8" s="1"/>
       <c r="E8" s="1"/>
-      <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
-      <c r="S8" s="1"/>
-    </row>
-    <row r="9" spans="1:19" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="C9" t="s">
+      <c r="R8" s="1"/>
+    </row>
+    <row r="9" spans="1:18" ht="48">
+      <c r="B9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9">
+        <v>2025</v>
+      </c>
+      <c r="D9" s="1" t="s">
         <v>41</v>
-      </c>
-      <c r="D9">
-        <v>2025</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>42</v>
@@ -814,98 +951,95 @@
       <c r="F9" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="1">
+        <v>30</v>
+      </c>
+      <c r="H9" s="1">
+        <v>10</v>
+      </c>
+      <c r="I9" s="1">
+        <v>20</v>
+      </c>
+      <c r="R9" t="s">
         <v>44</v>
       </c>
-      <c r="H9" s="1">
-        <v>30</v>
-      </c>
-      <c r="I9" s="1">
-        <v>10</v>
-      </c>
-      <c r="J9" s="1">
-        <v>20</v>
-      </c>
-      <c r="S9" t="s">
+    </row>
+    <row r="10" spans="1:18" ht="48">
+      <c r="B10" s="1" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="10" spans="1:19" ht="43.2" x14ac:dyDescent="0.3">
-      <c r="C10" t="s">
+      <c r="C10">
+        <v>2026</v>
+      </c>
+      <c r="D10" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="D10">
-        <v>2026</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>47</v>
       </c>
       <c r="F10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G10" s="1">
+        <v>13</v>
+      </c>
+      <c r="H10" s="1">
+        <v>5</v>
+      </c>
+      <c r="I10" s="1">
+        <v>8</v>
+      </c>
+      <c r="R10" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="G10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H10" s="1">
-        <v>13</v>
-      </c>
-      <c r="I10" s="1">
-        <v>5</v>
-      </c>
-      <c r="J10" s="1">
-        <v>8</v>
-      </c>
-      <c r="S10" s="1" t="s">
+    </row>
+    <row r="11" spans="1:18" ht="82.5" customHeight="1">
+      <c r="B11" s="1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="11" spans="1:19" ht="82.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C11" t="s">
+      <c r="C11">
+        <v>2024</v>
+      </c>
+      <c r="D11" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D11">
-        <v>2024</v>
-      </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>51</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="1">
+        <v>30</v>
+      </c>
+      <c r="H11" s="1">
+        <v>14</v>
+      </c>
+      <c r="I11" s="1">
+        <v>16</v>
+      </c>
+      <c r="J11" t="s">
         <v>53</v>
       </c>
-      <c r="H11" s="1">
-        <v>30</v>
-      </c>
-      <c r="I11" s="1">
-        <v>14</v>
-      </c>
-      <c r="J11" s="1">
-        <v>16</v>
-      </c>
-      <c r="K11" t="s">
+      <c r="K11" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="L11" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="M11" s="3" t="s">
+      <c r="R11" s="1" t="s">
         <v>56</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>57</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="S4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="R5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="S5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="S9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="S10" r:id="rId6" location="Bib1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="S11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="R3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="R4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="Q5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="R5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="R9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="R10" r:id="rId6" location="Bib1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="R11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -914,39 +1048,1351 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K1"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:J51"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.5" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="8" max="8" width="24.33203125" customWidth="1"/>
+    <col min="9" max="9" width="19.33203125" customWidth="1"/>
+    <col min="10" max="10" width="19.83203125" customWidth="1"/>
+    <col min="14" max="14" width="8.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10" s="5" customFormat="1">
+      <c r="A1" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="5" t="s">
+        <v>92</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" ht="16">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>31</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2">
+        <v>67</v>
+      </c>
+      <c r="E2">
+        <v>1.66</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2" t="s">
+        <v>90</v>
+      </c>
+      <c r="H2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
+        <v>48</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D3">
+        <v>65.400000000000006</v>
+      </c>
+      <c r="E3">
+        <v>1.64</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="16">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>28</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4">
+        <v>50</v>
+      </c>
+      <c r="E4">
+        <v>1.56</v>
+      </c>
+      <c r="F4">
+        <v>1</v>
+      </c>
+      <c r="G4" t="s">
+        <v>90</v>
+      </c>
+      <c r="H4" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
+        <v>23</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5">
+        <v>72.5</v>
+      </c>
+      <c r="E5">
+        <v>1.77</v>
+      </c>
+      <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>25</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6">
+        <v>73.5</v>
+      </c>
+      <c r="E6">
+        <v>1.83</v>
+      </c>
+      <c r="F6">
+        <v>1</v>
+      </c>
+      <c r="G6" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>23</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7">
+        <v>73</v>
+      </c>
+      <c r="E7">
+        <v>1.76</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H7" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="16">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>44</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D8">
         <v>65</v>
       </c>
-      <c r="J1" t="s">
-        <v>66</v>
-      </c>
-      <c r="K1" t="s">
-        <v>67</v>
+      <c r="E8">
+        <v>1.69</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8" t="s">
+        <v>90</v>
+      </c>
+      <c r="H8" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="16">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>30</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D9">
+        <v>57.1</v>
+      </c>
+      <c r="E9">
+        <v>1.66</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="16">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>57</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D10">
+        <v>86</v>
+      </c>
+      <c r="E10">
+        <v>1.88</v>
+      </c>
+      <c r="F10">
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>59</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D11">
+        <v>63.4</v>
+      </c>
+      <c r="E11">
+        <v>1.8</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="16">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12">
+        <v>26</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D12">
+        <v>61.3</v>
+      </c>
+      <c r="E12">
+        <v>1.7</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>90</v>
+      </c>
+      <c r="H12" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="16">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13">
+        <v>29</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D13">
+        <v>92</v>
+      </c>
+      <c r="E13">
+        <v>1.8</v>
+      </c>
+      <c r="F13">
+        <v>1</v>
+      </c>
+      <c r="G13" t="s">
+        <v>90</v>
+      </c>
+      <c r="H13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="16">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14">
+        <v>22</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14">
+        <v>67</v>
+      </c>
+      <c r="E14">
+        <v>1.58</v>
+      </c>
+      <c r="F14">
+        <v>1</v>
+      </c>
+      <c r="G14" t="s">
+        <v>90</v>
+      </c>
+      <c r="H14" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="16">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15">
+        <v>26</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15">
+        <v>73.8</v>
+      </c>
+      <c r="E15">
+        <v>1.76</v>
+      </c>
+      <c r="F15">
+        <v>1</v>
+      </c>
+      <c r="G15" t="s">
+        <v>90</v>
+      </c>
+      <c r="H15" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" ht="16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16">
+        <v>48</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D16">
+        <v>59.8</v>
+      </c>
+      <c r="E16">
+        <v>1.71</v>
+      </c>
+      <c r="F16">
+        <v>1</v>
+      </c>
+      <c r="G16" t="s">
+        <v>90</v>
+      </c>
+      <c r="H16" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="16">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17">
+        <v>33</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D17">
+        <v>87.5</v>
+      </c>
+      <c r="E17">
+        <v>1.92</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>90</v>
+      </c>
+      <c r="H17" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="16">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18">
+        <v>31</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D18">
+        <v>80.5</v>
+      </c>
+      <c r="E18">
+        <v>1.66</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="16">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19">
+        <v>38</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19">
+        <v>89.9</v>
+      </c>
+      <c r="E19">
+        <v>1.89</v>
+      </c>
+      <c r="F19">
+        <v>1</v>
+      </c>
+      <c r="G19" t="s">
+        <v>90</v>
+      </c>
+      <c r="H19" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="16">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20">
+        <v>62</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20">
+        <v>60.7</v>
+      </c>
+      <c r="E20">
+        <v>1.7</v>
+      </c>
+      <c r="F20">
+        <v>1</v>
+      </c>
+      <c r="G20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H20" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="16">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21">
+        <v>21</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D21">
+        <v>67.2</v>
+      </c>
+      <c r="E21">
+        <v>1.77</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H21" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="16">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22">
+        <v>24</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D22">
+        <v>63.5</v>
+      </c>
+      <c r="E22">
+        <v>1.6</v>
+      </c>
+      <c r="F22">
+        <v>1</v>
+      </c>
+      <c r="G22" t="s">
+        <v>90</v>
+      </c>
+      <c r="H22" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="16">
+      <c r="A23">
+        <v>22</v>
+      </c>
+      <c r="B23">
+        <v>21</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D23">
+        <v>89.6</v>
+      </c>
+      <c r="E23">
+        <v>1.84</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H23" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="16">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24">
+        <v>19</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D24">
+        <v>56.5</v>
+      </c>
+      <c r="E24">
+        <v>1.55</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>90</v>
+      </c>
+      <c r="H24" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="16">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25">
+        <v>40</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D25">
+        <v>61.8</v>
+      </c>
+      <c r="E25">
+        <v>1.65</v>
+      </c>
+      <c r="F25">
+        <v>1</v>
+      </c>
+      <c r="G25" t="s">
+        <v>90</v>
+      </c>
+      <c r="H25" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="16">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26">
+        <v>40</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D26">
+        <v>61.5</v>
+      </c>
+      <c r="E26">
+        <v>1.64</v>
+      </c>
+      <c r="F26">
+        <v>1</v>
+      </c>
+      <c r="G26" t="s">
+        <v>90</v>
+      </c>
+      <c r="H26" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" ht="16">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27">
+        <v>32</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D27">
+        <v>72.2</v>
+      </c>
+      <c r="E27">
+        <v>1.74</v>
+      </c>
+      <c r="F27">
+        <v>1</v>
+      </c>
+      <c r="G27" t="s">
+        <v>90</v>
+      </c>
+      <c r="H27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" ht="16">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28">
+        <v>28</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28">
+        <v>61.9</v>
+      </c>
+      <c r="E28">
+        <v>1.64</v>
+      </c>
+      <c r="F28">
+        <v>1</v>
+      </c>
+      <c r="G28" t="s">
+        <v>90</v>
+      </c>
+      <c r="H28" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" ht="16">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29">
+        <v>25</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D29">
+        <v>88</v>
+      </c>
+      <c r="E29">
+        <v>1.91</v>
+      </c>
+      <c r="F29">
+        <v>1</v>
+      </c>
+      <c r="G29" t="s">
+        <v>90</v>
+      </c>
+      <c r="H29" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="16">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30">
+        <v>25</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30">
+        <v>79.5</v>
+      </c>
+      <c r="E30">
+        <v>1.82</v>
+      </c>
+      <c r="F30">
+        <v>1</v>
+      </c>
+      <c r="G30" t="s">
+        <v>90</v>
+      </c>
+      <c r="H30" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="16">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31">
+        <v>21</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31">
+        <v>62.8</v>
+      </c>
+      <c r="E31">
+        <v>1.72</v>
+      </c>
+      <c r="F31">
+        <v>1</v>
+      </c>
+      <c r="G31" t="s">
+        <v>90</v>
+      </c>
+      <c r="H31" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" ht="16">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32">
+        <v>39</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32">
+        <v>74</v>
+      </c>
+      <c r="E32">
+        <v>1.74</v>
+      </c>
+      <c r="F32">
+        <v>1</v>
+      </c>
+      <c r="G32" t="s">
+        <v>90</v>
+      </c>
+      <c r="H32" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" ht="16">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33">
+        <v>52</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D33">
+        <v>87.2</v>
+      </c>
+      <c r="E33">
+        <v>1.77</v>
+      </c>
+      <c r="F33">
+        <v>1</v>
+      </c>
+      <c r="G33" t="s">
+        <v>90</v>
+      </c>
+      <c r="H33" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" ht="16">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34">
+        <v>35</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D34">
+        <v>62</v>
+      </c>
+      <c r="E34">
+        <v>1.7</v>
+      </c>
+      <c r="F34">
+        <v>1</v>
+      </c>
+      <c r="G34" t="s">
+        <v>90</v>
+      </c>
+      <c r="H34" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" ht="16">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35">
+        <v>48</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D35">
+        <v>89.4</v>
+      </c>
+      <c r="E35">
+        <v>1.9</v>
+      </c>
+      <c r="F35">
+        <v>1</v>
+      </c>
+      <c r="G35" t="s">
+        <v>90</v>
+      </c>
+      <c r="H35" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" ht="16">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36">
+        <v>63</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D36">
+        <v>60.2</v>
+      </c>
+      <c r="E36">
+        <v>1.66</v>
+      </c>
+      <c r="F36">
+        <v>1</v>
+      </c>
+      <c r="G36" t="s">
+        <v>90</v>
+      </c>
+      <c r="H36" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" ht="16">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37">
+        <v>58</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D37">
+        <v>73</v>
+      </c>
+      <c r="E37">
+        <v>1.69</v>
+      </c>
+      <c r="F37">
+        <v>1</v>
+      </c>
+      <c r="G37" t="s">
+        <v>90</v>
+      </c>
+      <c r="H37" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" ht="16">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38">
+        <v>50</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38">
+        <v>68</v>
+      </c>
+      <c r="E38">
+        <v>1.73</v>
+      </c>
+      <c r="F38">
+        <v>1</v>
+      </c>
+      <c r="G38" t="s">
+        <v>90</v>
+      </c>
+      <c r="H38" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" ht="16">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39">
+        <v>46</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D39">
+        <v>76</v>
+      </c>
+      <c r="E39">
+        <v>1.69</v>
+      </c>
+      <c r="F39">
+        <v>1</v>
+      </c>
+      <c r="G39" t="s">
+        <v>90</v>
+      </c>
+      <c r="H39" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" ht="16">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40">
+        <v>41</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D40">
+        <v>60.5</v>
+      </c>
+      <c r="E40">
+        <v>1.67</v>
+      </c>
+      <c r="F40">
+        <v>1</v>
+      </c>
+      <c r="G40" t="s">
+        <v>90</v>
+      </c>
+      <c r="H40" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" ht="16">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41">
+        <v>43</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D41">
+        <v>95</v>
+      </c>
+      <c r="E41">
+        <v>1.79</v>
+      </c>
+      <c r="F41">
+        <v>1</v>
+      </c>
+      <c r="G41" t="s">
+        <v>90</v>
+      </c>
+      <c r="H41" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" ht="16">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42">
+        <v>30</v>
+      </c>
+      <c r="C42" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D42">
+        <v>58</v>
+      </c>
+      <c r="E42">
+        <v>1.69</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42" t="s">
+        <v>90</v>
+      </c>
+      <c r="H42" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" ht="16">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43">
+        <v>64</v>
+      </c>
+      <c r="C43" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="D43">
+        <v>51.5</v>
+      </c>
+      <c r="E43">
+        <v>1.71</v>
+      </c>
+      <c r="F43">
+        <v>1</v>
+      </c>
+      <c r="G43" t="s">
+        <v>90</v>
+      </c>
+      <c r="H43" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" ht="16">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44">
+        <v>51</v>
+      </c>
+      <c r="C44" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D44">
+        <v>65.5</v>
+      </c>
+      <c r="E44">
+        <v>1.72</v>
+      </c>
+      <c r="F44">
+        <v>1</v>
+      </c>
+      <c r="G44" t="s">
+        <v>90</v>
+      </c>
+      <c r="H44" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" ht="16">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45">
+        <v>24</v>
+      </c>
+      <c r="C45" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D45">
+        <v>86</v>
+      </c>
+      <c r="E45">
+        <v>1.87</v>
+      </c>
+      <c r="F45">
+        <v>1</v>
+      </c>
+      <c r="G45" t="s">
+        <v>90</v>
+      </c>
+      <c r="H45" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" ht="16">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46">
+        <v>26</v>
+      </c>
+      <c r="C46" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D46">
+        <v>50.8</v>
+      </c>
+      <c r="E46">
+        <v>1.72</v>
+      </c>
+      <c r="F46">
+        <v>1</v>
+      </c>
+      <c r="G46" t="s">
+        <v>90</v>
+      </c>
+      <c r="H46" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" ht="16">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47">
+        <v>38</v>
+      </c>
+      <c r="C47" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D47">
+        <v>81.5</v>
+      </c>
+      <c r="E47">
+        <v>1.77</v>
+      </c>
+      <c r="F47">
+        <v>1</v>
+      </c>
+      <c r="G47" t="s">
+        <v>90</v>
+      </c>
+      <c r="H47" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" ht="16">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48">
+        <v>42</v>
+      </c>
+      <c r="C48" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D48">
+        <v>66.099999999999994</v>
+      </c>
+      <c r="E48">
+        <v>1.76</v>
+      </c>
+      <c r="F48">
+        <v>1</v>
+      </c>
+      <c r="G48" t="s">
+        <v>90</v>
+      </c>
+      <c r="H48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" ht="16">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49">
+        <v>31</v>
+      </c>
+      <c r="C49" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D49">
+        <v>74.8</v>
+      </c>
+      <c r="E49">
+        <v>1.88</v>
+      </c>
+      <c r="F49">
+        <v>1</v>
+      </c>
+      <c r="G49" t="s">
+        <v>90</v>
+      </c>
+      <c r="H49" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" ht="16">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50">
+        <v>67</v>
+      </c>
+      <c r="C50" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D50">
+        <v>98</v>
+      </c>
+      <c r="E50">
+        <v>1.83</v>
+      </c>
+      <c r="F50">
+        <v>1</v>
+      </c>
+      <c r="G50" t="s">
+        <v>90</v>
+      </c>
+      <c r="H50" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" ht="16">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51">
+        <v>21</v>
+      </c>
+      <c r="C51" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D51">
+        <v>74</v>
+      </c>
+      <c r="E51">
+        <v>1.78</v>
+      </c>
+      <c r="F51">
+        <v>1</v>
+      </c>
+      <c r="G51" t="s">
+        <v>90</v>
+      </c>
+      <c r="H51" t="s">
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -958,44 +2404,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
+    <col min="9" max="9" width="14.1640625" customWidth="1"/>
+    <col min="10" max="10" width="19.1640625" customWidth="1"/>
     <col min="11" max="11" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>61</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>64</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>65</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>66</v>
       </c>
-      <c r="K1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1003,7 +2451,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D2">
         <v>74</v>
@@ -1018,10 +2466,10 @@
         <v>21</v>
       </c>
       <c r="K2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1029,7 +2477,7 @@
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>72</v>
@@ -1047,7 +2495,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1055,7 +2503,7 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D4">
         <v>80</v>
@@ -1073,7 +2521,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1081,7 +2529,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>60</v>
@@ -1096,10 +2544,10 @@
         <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1107,7 +2555,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>71</v>
@@ -1122,7 +2570,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1130,7 +2578,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D7">
         <v>65</v>
@@ -1145,7 +2593,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1153,7 +2601,7 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D8">
         <v>72</v>
@@ -1168,7 +2616,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1176,7 +2624,7 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D9">
         <v>85</v>
@@ -1191,7 +2639,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1199,7 +2647,7 @@
         <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10">
         <v>76</v>
@@ -1214,7 +2662,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1222,7 +2670,7 @@
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D11">
         <v>80</v>
@@ -1240,7 +2688,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1248,7 +2696,7 @@
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D12">
         <v>75</v>
@@ -1263,10 +2711,10 @@
         <v>27</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1274,7 +2722,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D13">
         <v>80</v>
@@ -1289,7 +2737,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1297,7 +2745,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D14">
         <v>58</v>
@@ -1321,58 +2769,58 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="11" max="11" width="19.109375" customWidth="1"/>
+    <col min="11" max="11" width="19.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>61</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>64</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>65</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>66</v>
       </c>
-      <c r="K1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -1381,21 +2829,21 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1404,21 +2852,21 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -1427,21 +2875,21 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -1450,21 +2898,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -1473,21 +2921,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -1496,21 +2944,21 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -1519,21 +2967,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -1542,21 +2990,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -1565,21 +3013,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E11" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1597,52 +3045,52 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
         <v>58</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>59</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>61</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>64</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>65</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>66</v>
       </c>
-      <c r="K1" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C2" t="s">
         <v>72</v>
-      </c>
-      <c r="C2" t="s">
-        <v>73</v>
       </c>
       <c r="D2">
         <v>69.86</v>
@@ -1654,18 +3102,18 @@
         <v>3</v>
       </c>
       <c r="K2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D3">
         <v>66.680000000000007</v>
@@ -1677,18 +3125,18 @@
         <v>4</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
         <v>72</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
       </c>
       <c r="D4">
         <v>53.07</v>
@@ -1700,18 +3148,18 @@
         <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D5">
         <v>71.67</v>
@@ -1723,15 +3171,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D6">
         <v>90.7</v>
@@ -1743,15 +3191,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" t="s">
         <v>72</v>
-      </c>
-      <c r="C7" t="s">
-        <v>73</v>
       </c>
       <c r="D7">
         <v>48.99</v>
@@ -1763,15 +3211,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>71</v>
+      </c>
+      <c r="C8" t="s">
         <v>72</v>
-      </c>
-      <c r="C8" t="s">
-        <v>73</v>
       </c>
       <c r="D8">
         <v>63.96</v>

</xml_diff>

<commit_message>
Update database_inventory DB1 sheet
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/user/TeamProject/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF009508-D356-0346-BFB3-6CF22E7AFCF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE757F6-8ABE-4F17-9A9B-888006D49CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="27420" windowHeight="17500" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36" yWindow="0" windowWidth="14724" windowHeight="12336" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="90">
   <si>
     <t>Database No.</t>
   </si>
@@ -337,21 +337,12 @@
   <si>
     <t>W</t>
   </si>
-  <si>
-    <t xml:space="preserve">C1-C5 variable trails </t>
-  </si>
-  <si>
-    <t>only C4 &amp; C5 (variable trials)</t>
-  </si>
-  <si>
-    <t>Duration per trials(s)</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -400,13 +391,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -441,7 +425,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -454,13 +438,10 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -657,81 +638,81 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="11.83203125" customWidth="1"/>
-    <col min="2" max="2" width="12.5" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.1640625" customWidth="1"/>
-    <col min="4" max="4" width="33.83203125" customWidth="1"/>
+    <col min="1" max="1" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.109375" customWidth="1"/>
+    <col min="4" max="4" width="33.77734375" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="23.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.5" customWidth="1"/>
-    <col min="9" max="9" width="9.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.44140625" customWidth="1"/>
+    <col min="9" max="9" width="9.77734375" customWidth="1"/>
     <col min="10" max="10" width="12.6640625" customWidth="1"/>
     <col min="11" max="11" width="14.33203125" customWidth="1"/>
     <col min="12" max="12" width="12.6640625" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="28.5" customWidth="1"/>
-    <col min="15" max="15" width="24.5" customWidth="1"/>
+    <col min="14" max="14" width="28.44140625" customWidth="1"/>
+    <col min="15" max="15" width="24.44140625" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
-    <col min="17" max="17" width="40.83203125" style="1" customWidth="1"/>
-    <col min="18" max="18" width="29.83203125" customWidth="1"/>
+    <col min="17" max="17" width="40.77734375" style="1" customWidth="1"/>
+    <col min="18" max="18" width="29.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="6" customFormat="1" ht="17">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:18" s="5" customFormat="1" ht="15.6">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="B1" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="6" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="6" t="s">
+      <c r="I1" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="6" t="s">
+      <c r="K1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="6" t="s">
+      <c r="L1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="6" t="s">
+      <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="6" t="s">
+      <c r="O1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="6" t="s">
+      <c r="P1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="64">
+    <row r="2" spans="1:18" ht="43.2">
       <c r="A2">
         <v>1</v>
       </c>
@@ -784,7 +765,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="48">
+    <row r="3" spans="1:18" ht="43.2">
       <c r="A3">
         <v>2</v>
       </c>
@@ -828,7 +809,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="51">
+    <row r="4" spans="1:18" ht="46.8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -872,7 +853,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="48">
+    <row r="5" spans="1:18" ht="43.2">
       <c r="A5">
         <v>4</v>
       </c>
@@ -935,7 +916,7 @@
       <c r="I8" s="1"/>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" ht="48">
+    <row r="9" spans="1:18" ht="57.6">
       <c r="B9" s="1" t="s">
         <v>40</v>
       </c>
@@ -964,7 +945,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="48">
+    <row r="10" spans="1:18" ht="43.2">
       <c r="B10" s="1" t="s">
         <v>45</v>
       </c>
@@ -1048,61 +1029,61 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J51"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <dimension ref="A1:K51"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" customWidth="1"/>
-    <col min="3" max="3" width="10.5" customWidth="1"/>
+    <col min="2" max="2" width="10.77734375" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
-    <col min="7" max="7" width="16.6640625" customWidth="1"/>
-    <col min="8" max="8" width="24.33203125" customWidth="1"/>
-    <col min="9" max="9" width="19.33203125" customWidth="1"/>
-    <col min="10" max="10" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="8.83203125" customWidth="1"/>
+    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="8" max="8" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="24.33203125" customWidth="1"/>
+    <col min="10" max="10" width="19.33203125" customWidth="1"/>
+    <col min="11" max="11" width="19.77734375" customWidth="1"/>
+    <col min="15" max="15" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="5" customFormat="1">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:11">
+      <c r="A1" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" t="s">
         <v>59</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" t="s">
         <v>61</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="G1" t="s">
         <v>62</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="H1" t="s">
         <v>63</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="I1" t="s">
         <v>64</v>
       </c>
-      <c r="I1" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" t="s">
+        <v>65</v>
+      </c>
+      <c r="K1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="16">
+    <row r="2" spans="1:11">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>31</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D2">
@@ -1111,24 +1092,21 @@
       <c r="E2">
         <v>1.66</v>
       </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" ht="16">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
         <v>48</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D3">
@@ -1137,24 +1115,21 @@
       <c r="E3">
         <v>1.64</v>
       </c>
-      <c r="F3">
-        <v>1</v>
-      </c>
-      <c r="G3" t="s">
-        <v>90</v>
-      </c>
-      <c r="H3" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" ht="16">
+      <c r="G3">
+        <v>1</v>
+      </c>
+      <c r="H3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
         <v>28</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D4">
@@ -1163,24 +1138,21 @@
       <c r="E4">
         <v>1.56</v>
       </c>
-      <c r="F4">
-        <v>1</v>
-      </c>
-      <c r="G4" t="s">
-        <v>90</v>
-      </c>
-      <c r="H4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" ht="16">
+      <c r="G4">
+        <v>1</v>
+      </c>
+      <c r="H4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5">
         <v>23</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C5" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D5">
@@ -1189,24 +1161,21 @@
       <c r="E5">
         <v>1.77</v>
       </c>
-      <c r="F5">
-        <v>1</v>
-      </c>
-      <c r="G5" t="s">
-        <v>90</v>
-      </c>
-      <c r="H5" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" ht="16">
+      <c r="G5">
+        <v>1</v>
+      </c>
+      <c r="H5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6">
         <v>25</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C6" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D6">
@@ -1215,24 +1184,21 @@
       <c r="E6">
         <v>1.83</v>
       </c>
-      <c r="F6">
-        <v>1</v>
-      </c>
-      <c r="G6" t="s">
-        <v>90</v>
-      </c>
-      <c r="H6" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="16">
+      <c r="G6">
+        <v>0</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7">
         <v>23</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D7">
@@ -1241,24 +1207,21 @@
       <c r="E7">
         <v>1.76</v>
       </c>
-      <c r="F7">
-        <v>1</v>
-      </c>
-      <c r="G7" t="s">
-        <v>90</v>
-      </c>
-      <c r="H7" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="16">
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8">
         <v>44</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D8">
@@ -1267,24 +1230,21 @@
       <c r="E8">
         <v>1.69</v>
       </c>
-      <c r="F8">
-        <v>1</v>
-      </c>
-      <c r="G8" t="s">
-        <v>90</v>
-      </c>
-      <c r="H8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="16">
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9">
         <v>30</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D9">
@@ -1293,24 +1253,21 @@
       <c r="E9">
         <v>1.66</v>
       </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="G9" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" ht="16">
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10">
         <v>57</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D10">
@@ -1319,24 +1276,21 @@
       <c r="E10">
         <v>1.88</v>
       </c>
-      <c r="F10">
-        <v>1</v>
-      </c>
-      <c r="G10" t="s">
-        <v>90</v>
-      </c>
-      <c r="H10" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="16">
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11">
         <v>59</v>
       </c>
-      <c r="C11" s="8" t="s">
+      <c r="C11" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D11">
@@ -1345,24 +1299,21 @@
       <c r="E11">
         <v>1.8</v>
       </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="s">
-        <v>90</v>
-      </c>
-      <c r="H11" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" ht="16">
+      <c r="G11">
+        <v>1</v>
+      </c>
+      <c r="H11">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12">
         <v>26</v>
       </c>
-      <c r="C12" s="8" t="s">
+      <c r="C12" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D12">
@@ -1371,24 +1322,21 @@
       <c r="E12">
         <v>1.7</v>
       </c>
-      <c r="F12">
-        <v>1</v>
-      </c>
-      <c r="G12" t="s">
-        <v>90</v>
-      </c>
-      <c r="H12" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="16">
+      <c r="G12">
+        <v>1</v>
+      </c>
+      <c r="H12">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13">
         <v>29</v>
       </c>
-      <c r="C13" s="8" t="s">
+      <c r="C13" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D13">
@@ -1397,24 +1345,21 @@
       <c r="E13">
         <v>1.8</v>
       </c>
-      <c r="F13">
-        <v>1</v>
-      </c>
-      <c r="G13" t="s">
-        <v>90</v>
-      </c>
-      <c r="H13" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="16">
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14">
         <v>22</v>
       </c>
-      <c r="C14" s="8" t="s">
+      <c r="C14" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D14">
@@ -1423,24 +1368,21 @@
       <c r="E14">
         <v>1.58</v>
       </c>
-      <c r="F14">
-        <v>1</v>
-      </c>
-      <c r="G14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H14" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="16">
+      <c r="G14">
+        <v>0</v>
+      </c>
+      <c r="H14">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15">
         <v>26</v>
       </c>
-      <c r="C15" s="8" t="s">
+      <c r="C15" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D15">
@@ -1449,24 +1391,21 @@
       <c r="E15">
         <v>1.76</v>
       </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-      <c r="G15" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="16" spans="1:10" ht="16">
+      <c r="G15">
+        <v>1</v>
+      </c>
+      <c r="H15">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16">
         <v>48</v>
       </c>
-      <c r="C16" s="8" t="s">
+      <c r="C16" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D16">
@@ -1475,24 +1414,21 @@
       <c r="E16">
         <v>1.71</v>
       </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-      <c r="G16" t="s">
-        <v>90</v>
-      </c>
-      <c r="H16" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" ht="16">
+      <c r="G16">
+        <v>1</v>
+      </c>
+      <c r="H16">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17">
         <v>33</v>
       </c>
-      <c r="C17" s="8" t="s">
+      <c r="C17" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D17">
@@ -1501,24 +1437,21 @@
       <c r="E17">
         <v>1.92</v>
       </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17" t="s">
-        <v>90</v>
-      </c>
-      <c r="H17" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" ht="16">
+      <c r="G17">
+        <v>1</v>
+      </c>
+      <c r="H17">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18">
         <v>31</v>
       </c>
-      <c r="C18" s="8" t="s">
+      <c r="C18" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D18">
@@ -1527,24 +1460,21 @@
       <c r="E18">
         <v>1.66</v>
       </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-      <c r="G18" t="s">
-        <v>90</v>
-      </c>
-      <c r="H18" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="16">
+      <c r="G18">
+        <v>1</v>
+      </c>
+      <c r="H18">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19">
         <v>38</v>
       </c>
-      <c r="C19" s="8" t="s">
+      <c r="C19" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D19">
@@ -1553,24 +1483,21 @@
       <c r="E19">
         <v>1.89</v>
       </c>
-      <c r="F19">
-        <v>1</v>
-      </c>
-      <c r="G19" t="s">
-        <v>90</v>
-      </c>
-      <c r="H19" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8" ht="16">
+      <c r="G19">
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20">
         <v>62</v>
       </c>
-      <c r="C20" s="8" t="s">
+      <c r="C20" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D20">
@@ -1579,24 +1506,21 @@
       <c r="E20">
         <v>1.7</v>
       </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-      <c r="G20" t="s">
-        <v>90</v>
-      </c>
-      <c r="H20" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8" ht="16">
+      <c r="G20">
+        <v>1</v>
+      </c>
+      <c r="H20">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21">
         <v>21</v>
       </c>
-      <c r="C21" s="8" t="s">
+      <c r="C21" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D21">
@@ -1605,24 +1529,21 @@
       <c r="E21">
         <v>1.77</v>
       </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-      <c r="G21" t="s">
-        <v>90</v>
-      </c>
-      <c r="H21" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8" ht="16">
+      <c r="G21">
+        <v>1</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22">
         <v>24</v>
       </c>
-      <c r="C22" s="8" t="s">
+      <c r="C22" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D22">
@@ -1631,24 +1552,21 @@
       <c r="E22">
         <v>1.6</v>
       </c>
-      <c r="F22">
-        <v>1</v>
-      </c>
-      <c r="G22" t="s">
-        <v>90</v>
-      </c>
-      <c r="H22" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" ht="16">
+      <c r="G22">
+        <v>1</v>
+      </c>
+      <c r="H22">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23">
         <v>21</v>
       </c>
-      <c r="C23" s="8" t="s">
+      <c r="C23" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D23">
@@ -1657,24 +1575,21 @@
       <c r="E23">
         <v>1.84</v>
       </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-      <c r="G23" t="s">
-        <v>90</v>
-      </c>
-      <c r="H23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8" ht="16">
+      <c r="G23">
+        <v>1</v>
+      </c>
+      <c r="H23">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24">
         <v>19</v>
       </c>
-      <c r="C24" s="8" t="s">
+      <c r="C24" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D24">
@@ -1683,24 +1598,21 @@
       <c r="E24">
         <v>1.55</v>
       </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-      <c r="G24" t="s">
-        <v>90</v>
-      </c>
-      <c r="H24" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8" ht="16">
+      <c r="G24">
+        <v>1</v>
+      </c>
+      <c r="H24">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25">
         <v>40</v>
       </c>
-      <c r="C25" s="8" t="s">
+      <c r="C25" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D25">
@@ -1709,24 +1621,21 @@
       <c r="E25">
         <v>1.65</v>
       </c>
-      <c r="F25">
-        <v>1</v>
-      </c>
-      <c r="G25" t="s">
-        <v>90</v>
-      </c>
-      <c r="H25" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" ht="16">
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26">
         <v>40</v>
       </c>
-      <c r="C26" s="8" t="s">
+      <c r="C26" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D26">
@@ -1735,24 +1644,21 @@
       <c r="E26">
         <v>1.64</v>
       </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-      <c r="G26" t="s">
-        <v>90</v>
-      </c>
-      <c r="H26" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" ht="16">
+      <c r="G26">
+        <v>1</v>
+      </c>
+      <c r="H26">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27">
         <v>32</v>
       </c>
-      <c r="C27" s="8" t="s">
+      <c r="C27" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D27">
@@ -1761,24 +1667,21 @@
       <c r="E27">
         <v>1.74</v>
       </c>
-      <c r="F27">
-        <v>1</v>
-      </c>
-      <c r="G27" t="s">
-        <v>90</v>
-      </c>
-      <c r="H27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" ht="16">
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28">
         <v>28</v>
       </c>
-      <c r="C28" s="8" t="s">
+      <c r="C28" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D28">
@@ -1787,24 +1690,21 @@
       <c r="E28">
         <v>1.64</v>
       </c>
-      <c r="F28">
-        <v>1</v>
-      </c>
-      <c r="G28" t="s">
-        <v>90</v>
-      </c>
-      <c r="H28" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" ht="16">
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29">
         <v>25</v>
       </c>
-      <c r="C29" s="8" t="s">
+      <c r="C29" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D29">
@@ -1813,24 +1713,21 @@
       <c r="E29">
         <v>1.91</v>
       </c>
-      <c r="F29">
-        <v>1</v>
-      </c>
-      <c r="G29" t="s">
-        <v>90</v>
-      </c>
-      <c r="H29" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" ht="16">
+      <c r="G29">
+        <v>1</v>
+      </c>
+      <c r="H29">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30">
         <v>25</v>
       </c>
-      <c r="C30" s="8" t="s">
+      <c r="C30" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D30">
@@ -1839,24 +1736,21 @@
       <c r="E30">
         <v>1.82</v>
       </c>
-      <c r="F30">
-        <v>1</v>
-      </c>
-      <c r="G30" t="s">
-        <v>90</v>
-      </c>
-      <c r="H30" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" ht="16">
+      <c r="G30">
+        <v>1</v>
+      </c>
+      <c r="H30">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31">
         <v>21</v>
       </c>
-      <c r="C31" s="8" t="s">
+      <c r="C31" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D31">
@@ -1865,24 +1759,21 @@
       <c r="E31">
         <v>1.72</v>
       </c>
-      <c r="F31">
-        <v>1</v>
-      </c>
-      <c r="G31" t="s">
-        <v>90</v>
-      </c>
-      <c r="H31" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" ht="16">
+      <c r="G31">
+        <v>1</v>
+      </c>
+      <c r="H31">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32">
         <v>39</v>
       </c>
-      <c r="C32" s="8" t="s">
+      <c r="C32" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D32">
@@ -1891,24 +1782,21 @@
       <c r="E32">
         <v>1.74</v>
       </c>
-      <c r="F32">
-        <v>1</v>
-      </c>
-      <c r="G32" t="s">
-        <v>90</v>
-      </c>
-      <c r="H32" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" ht="16">
+      <c r="G32">
+        <v>1</v>
+      </c>
+      <c r="H32">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33">
         <v>52</v>
       </c>
-      <c r="C33" s="8" t="s">
+      <c r="C33" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D33">
@@ -1917,24 +1805,21 @@
       <c r="E33">
         <v>1.77</v>
       </c>
-      <c r="F33">
-        <v>1</v>
-      </c>
-      <c r="G33" t="s">
-        <v>90</v>
-      </c>
-      <c r="H33" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" ht="16">
+      <c r="G33">
+        <v>0</v>
+      </c>
+      <c r="H33">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34">
         <v>35</v>
       </c>
-      <c r="C34" s="8" t="s">
+      <c r="C34" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D34">
@@ -1943,24 +1828,21 @@
       <c r="E34">
         <v>1.7</v>
       </c>
-      <c r="F34">
-        <v>1</v>
-      </c>
-      <c r="G34" t="s">
-        <v>90</v>
-      </c>
-      <c r="H34" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" ht="16">
+      <c r="G34">
+        <v>0</v>
+      </c>
+      <c r="H34">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35">
         <v>48</v>
       </c>
-      <c r="C35" s="8" t="s">
+      <c r="C35" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D35">
@@ -1969,24 +1851,21 @@
       <c r="E35">
         <v>1.9</v>
       </c>
-      <c r="F35">
-        <v>1</v>
-      </c>
-      <c r="G35" t="s">
-        <v>90</v>
-      </c>
-      <c r="H35" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" ht="16">
+      <c r="G35">
+        <v>1</v>
+      </c>
+      <c r="H35">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36">
         <v>63</v>
       </c>
-      <c r="C36" s="8" t="s">
+      <c r="C36" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D36">
@@ -1995,24 +1874,21 @@
       <c r="E36">
         <v>1.66</v>
       </c>
-      <c r="F36">
-        <v>1</v>
-      </c>
-      <c r="G36" t="s">
-        <v>90</v>
-      </c>
-      <c r="H36" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" ht="16">
+      <c r="G36">
+        <v>1</v>
+      </c>
+      <c r="H36">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37">
         <v>58</v>
       </c>
-      <c r="C37" s="8" t="s">
+      <c r="C37" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D37">
@@ -2021,24 +1897,21 @@
       <c r="E37">
         <v>1.69</v>
       </c>
-      <c r="F37">
-        <v>1</v>
-      </c>
-      <c r="G37" t="s">
-        <v>90</v>
-      </c>
-      <c r="H37" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" ht="16">
+      <c r="G37">
+        <v>1</v>
+      </c>
+      <c r="H37">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38">
         <v>50</v>
       </c>
-      <c r="C38" s="8" t="s">
+      <c r="C38" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D38">
@@ -2047,24 +1920,21 @@
       <c r="E38">
         <v>1.73</v>
       </c>
-      <c r="F38">
-        <v>1</v>
-      </c>
-      <c r="G38" t="s">
-        <v>90</v>
-      </c>
-      <c r="H38" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" ht="16">
+      <c r="G38">
+        <v>0</v>
+      </c>
+      <c r="H38">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39">
         <v>46</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D39">
@@ -2073,24 +1943,21 @@
       <c r="E39">
         <v>1.69</v>
       </c>
-      <c r="F39">
-        <v>1</v>
-      </c>
-      <c r="G39" t="s">
-        <v>90</v>
-      </c>
-      <c r="H39" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" ht="16">
+      <c r="G39">
+        <v>1</v>
+      </c>
+      <c r="H39">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40">
         <v>41</v>
       </c>
-      <c r="C40" s="8" t="s">
+      <c r="C40" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D40">
@@ -2099,24 +1966,21 @@
       <c r="E40">
         <v>1.67</v>
       </c>
-      <c r="F40">
-        <v>1</v>
-      </c>
-      <c r="G40" t="s">
-        <v>90</v>
-      </c>
-      <c r="H40" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" ht="16">
+      <c r="G40">
+        <v>1</v>
+      </c>
+      <c r="H40">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41">
         <v>43</v>
       </c>
-      <c r="C41" s="8" t="s">
+      <c r="C41" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D41">
@@ -2125,24 +1989,21 @@
       <c r="E41">
         <v>1.79</v>
       </c>
-      <c r="F41">
-        <v>1</v>
-      </c>
-      <c r="G41" t="s">
-        <v>90</v>
-      </c>
-      <c r="H41" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" ht="16">
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42">
         <v>30</v>
       </c>
-      <c r="C42" s="8" t="s">
+      <c r="C42" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D42">
@@ -2151,24 +2012,21 @@
       <c r="E42">
         <v>1.69</v>
       </c>
-      <c r="F42">
-        <v>1</v>
-      </c>
-      <c r="G42" t="s">
-        <v>90</v>
-      </c>
-      <c r="H42" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" ht="16">
+      <c r="G42">
+        <v>1</v>
+      </c>
+      <c r="H42">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43">
         <v>64</v>
       </c>
-      <c r="C43" s="8" t="s">
+      <c r="C43" s="7" t="s">
         <v>89</v>
       </c>
       <c r="D43">
@@ -2177,24 +2035,21 @@
       <c r="E43">
         <v>1.71</v>
       </c>
-      <c r="F43">
-        <v>1</v>
-      </c>
-      <c r="G43" t="s">
-        <v>90</v>
-      </c>
-      <c r="H43" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" ht="16">
+      <c r="G43">
+        <v>1</v>
+      </c>
+      <c r="H43">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44">
         <v>51</v>
       </c>
-      <c r="C44" s="8" t="s">
+      <c r="C44" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D44">
@@ -2203,24 +2058,21 @@
       <c r="E44">
         <v>1.72</v>
       </c>
-      <c r="F44">
-        <v>1</v>
-      </c>
-      <c r="G44" t="s">
-        <v>90</v>
-      </c>
-      <c r="H44" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" ht="16">
+      <c r="G44">
+        <v>1</v>
+      </c>
+      <c r="H44">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45">
         <v>24</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D45">
@@ -2229,24 +2081,21 @@
       <c r="E45">
         <v>1.87</v>
       </c>
-      <c r="F45">
-        <v>1</v>
-      </c>
-      <c r="G45" t="s">
-        <v>90</v>
-      </c>
-      <c r="H45" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" ht="16">
+      <c r="G45">
+        <v>1</v>
+      </c>
+      <c r="H45">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46">
         <v>26</v>
       </c>
-      <c r="C46" s="8" t="s">
+      <c r="C46" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D46">
@@ -2255,24 +2104,21 @@
       <c r="E46">
         <v>1.72</v>
       </c>
-      <c r="F46">
-        <v>1</v>
-      </c>
-      <c r="G46" t="s">
-        <v>90</v>
-      </c>
-      <c r="H46" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" ht="16">
+      <c r="G46">
+        <v>1</v>
+      </c>
+      <c r="H46">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47">
         <v>38</v>
       </c>
-      <c r="C47" s="8" t="s">
+      <c r="C47" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D47">
@@ -2281,24 +2127,21 @@
       <c r="E47">
         <v>1.77</v>
       </c>
-      <c r="F47">
-        <v>1</v>
-      </c>
-      <c r="G47" t="s">
-        <v>90</v>
-      </c>
-      <c r="H47" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" ht="16">
+      <c r="G47">
+        <v>1</v>
+      </c>
+      <c r="H47">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48">
         <v>42</v>
       </c>
-      <c r="C48" s="8" t="s">
+      <c r="C48" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D48">
@@ -2307,24 +2150,21 @@
       <c r="E48">
         <v>1.76</v>
       </c>
-      <c r="F48">
-        <v>1</v>
-      </c>
-      <c r="G48" t="s">
-        <v>90</v>
-      </c>
-      <c r="H48" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" ht="16">
+      <c r="G48">
+        <v>1</v>
+      </c>
+      <c r="H48">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49">
         <v>31</v>
       </c>
-      <c r="C49" s="8" t="s">
+      <c r="C49" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D49">
@@ -2333,24 +2173,21 @@
       <c r="E49">
         <v>1.88</v>
       </c>
-      <c r="F49">
-        <v>1</v>
-      </c>
-      <c r="G49" t="s">
-        <v>90</v>
-      </c>
-      <c r="H49" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" ht="16">
+      <c r="G49">
+        <v>1</v>
+      </c>
+      <c r="H49">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50">
         <v>67</v>
       </c>
-      <c r="C50" s="8" t="s">
+      <c r="C50" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D50">
@@ -2359,24 +2196,21 @@
       <c r="E50">
         <v>1.83</v>
       </c>
-      <c r="F50">
-        <v>1</v>
-      </c>
-      <c r="G50" t="s">
-        <v>90</v>
-      </c>
-      <c r="H50" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" ht="16">
+      <c r="G50">
+        <v>1</v>
+      </c>
+      <c r="H50">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51">
         <v>21</v>
       </c>
-      <c r="C51" s="8" t="s">
+      <c r="C51" s="7" t="s">
         <v>67</v>
       </c>
       <c r="D51">
@@ -2385,14 +2219,11 @@
       <c r="E51">
         <v>1.78</v>
       </c>
-      <c r="F51">
-        <v>1</v>
-      </c>
-      <c r="G51" t="s">
-        <v>90</v>
-      </c>
-      <c r="H51" t="s">
-        <v>91</v>
+      <c r="G51">
+        <v>0</v>
+      </c>
+      <c r="H51">
+        <v>10</v>
       </c>
     </row>
   </sheetData>
@@ -2404,10 +2235,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="9" max="9" width="14.1640625" customWidth="1"/>
-    <col min="10" max="10" width="19.1640625" customWidth="1"/>
+    <col min="9" max="9" width="14.109375" customWidth="1"/>
+    <col min="10" max="10" width="19.109375" customWidth="1"/>
     <col min="11" max="11" width="28.33203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2769,9 +2600,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="11" max="11" width="19.1640625" customWidth="1"/>
+    <col min="11" max="11" width="19.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -3045,7 +2876,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:K8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>

</xml_diff>

<commit_message>
Update database_inventory DB with error
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFE757F6-8ABE-4F17-9A9B-888006D49CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77ADC58E-6F4B-4E56-816D-9865C1EE2D88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36" yWindow="0" windowWidth="14724" windowHeight="12336" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,19 @@
     <sheet name="DB3" sheetId="4" r:id="rId4"/>
     <sheet name="DB4" sheetId="5" r:id="rId5"/>
   </sheets>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -254,9 +265,6 @@
     <t>M</t>
   </si>
   <si>
-    <t>3-all ('LoadingError')</t>
-  </si>
-  <si>
     <t>T04_Cal_relabeled (missing GRF)</t>
   </si>
   <si>
@@ -270,9 +278,6 @@
   </si>
   <si>
     <t>1:3 (No ID)</t>
-  </si>
-  <si>
-    <t>4 (First half No ID)</t>
   </si>
   <si>
     <t>T02_-130 (MarkerFitterError)</t>
@@ -336,6 +341,12 @@
   </si>
   <si>
     <t>W</t>
+  </si>
+  <si>
+    <t>4 (1st half No ID, 2nd half wrong)</t>
+  </si>
+  <si>
+    <t>3-all ('LoadingError'), 4 in total</t>
   </si>
 </sst>
 </file>
@@ -717,19 +728,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C2">
         <v>2019</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E2" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G2">
         <v>50</v>
@@ -741,28 +752,28 @@
         <v>26</v>
       </c>
       <c r="J2" t="s">
+        <v>80</v>
+      </c>
+      <c r="K2" t="s">
+        <v>81</v>
+      </c>
+      <c r="L2" t="s">
         <v>82</v>
       </c>
-      <c r="K2" t="s">
+      <c r="M2" t="s">
+        <v>84</v>
+      </c>
+      <c r="N2" t="s">
         <v>83</v>
       </c>
-      <c r="L2" t="s">
-        <v>84</v>
-      </c>
-      <c r="M2" t="s">
-        <v>86</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>85</v>
-      </c>
-      <c r="O2" t="s">
-        <v>87</v>
       </c>
       <c r="P2">
         <v>2</v>
       </c>
       <c r="Q2" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="43.2">
@@ -782,7 +793,7 @@
         <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="G3">
         <v>13</v>
@@ -826,7 +837,7 @@
         <v>19</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="G4" s="1">
         <v>10</v>
@@ -1107,7 +1118,7 @@
         <v>48</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D3">
         <v>65.400000000000006</v>
@@ -1130,7 +1141,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1222,7 +1233,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D8">
         <v>65</v>
@@ -1245,7 +1256,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D9">
         <v>57.1</v>
@@ -1314,7 +1325,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D12">
         <v>61.3</v>
@@ -1360,7 +1371,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D14">
         <v>67</v>
@@ -1383,7 +1394,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D15">
         <v>73.8</v>
@@ -1406,7 +1417,7 @@
         <v>48</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D16">
         <v>59.8</v>
@@ -1452,7 +1463,7 @@
         <v>31</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D18">
         <v>80.5</v>
@@ -1498,7 +1509,7 @@
         <v>62</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D20">
         <v>60.7</v>
@@ -1544,7 +1555,7 @@
         <v>24</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D22">
         <v>63.5</v>
@@ -1590,7 +1601,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D24">
         <v>56.5</v>
@@ -1613,7 +1624,7 @@
         <v>40</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D25">
         <v>61.8</v>
@@ -1636,7 +1647,7 @@
         <v>40</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D26">
         <v>61.5</v>
@@ -1682,7 +1693,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D28">
         <v>61.9</v>
@@ -1751,7 +1762,7 @@
         <v>21</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D31">
         <v>62.8</v>
@@ -1820,7 +1831,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D34">
         <v>62</v>
@@ -1866,7 +1877,7 @@
         <v>63</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D36">
         <v>60.2</v>
@@ -1889,7 +1900,7 @@
         <v>58</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D37">
         <v>73</v>
@@ -1912,7 +1923,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D38">
         <v>68</v>
@@ -1935,7 +1946,7 @@
         <v>46</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D39">
         <v>76</v>
@@ -1958,7 +1969,7 @@
         <v>41</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D40">
         <v>60.5</v>
@@ -2004,7 +2015,7 @@
         <v>30</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D42">
         <v>58</v>
@@ -2027,7 +2038,7 @@
         <v>64</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D43">
         <v>51.5</v>
@@ -2296,8 +2307,11 @@
       <c r="H2">
         <v>21</v>
       </c>
+      <c r="I2">
+        <v>17</v>
+      </c>
       <c r="K2" t="s">
-        <v>68</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2375,7 +2389,7 @@
         <v>17</v>
       </c>
       <c r="K5" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -2542,7 +2556,7 @@
         <v>27</v>
       </c>
       <c r="K12" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2642,16 +2656,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2665,16 +2679,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2688,16 +2702,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2711,16 +2725,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2734,16 +2748,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -2757,16 +2771,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -2780,16 +2794,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -2803,16 +2817,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -2826,16 +2840,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -2849,16 +2863,16 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -2918,10 +2932,10 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C2" t="s">
         <v>71</v>
-      </c>
-      <c r="C2" t="s">
-        <v>72</v>
       </c>
       <c r="D2">
         <v>69.86</v>
@@ -2932,8 +2946,11 @@
       <c r="H2">
         <v>3</v>
       </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
       <c r="K2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -2941,7 +2958,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C3" t="s">
         <v>67</v>
@@ -2955,8 +2972,11 @@
       <c r="H3">
         <v>4</v>
       </c>
+      <c r="I3">
+        <v>3</v>
+      </c>
       <c r="K3" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -2964,10 +2984,10 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C4" t="s">
         <v>71</v>
-      </c>
-      <c r="C4" t="s">
-        <v>72</v>
       </c>
       <c r="D4">
         <v>53.07</v>
@@ -2979,7 +2999,7 @@
         <v>3</v>
       </c>
       <c r="K4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -2987,7 +3007,7 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C5" t="s">
         <v>67</v>
@@ -3007,7 +3027,7 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C6" t="s">
         <v>67</v>
@@ -3027,10 +3047,10 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7" t="s">
         <v>71</v>
-      </c>
-      <c r="C7" t="s">
-        <v>72</v>
       </c>
       <c r="D7">
         <v>48.99</v>
@@ -3047,10 +3067,10 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" t="s">
         <v>71</v>
-      </c>
-      <c r="C8" t="s">
-        <v>72</v>
       </c>
       <c r="D8">
         <v>63.96</v>

</xml_diff>

<commit_message>
Update database_inventory table DB1 available files
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A9B790-7151-41C9-B567-910EE126AD07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F41193-90DF-484F-926D-B45044908842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="92">
   <si>
     <t>Database No.</t>
   </si>
@@ -347,6 +347,12 @@
   </si>
   <si>
     <t>3-all ('LoadingError'), 4 in total</t>
+  </si>
+  <si>
+    <t>Walk trials C4-C5 (files)</t>
+  </si>
+  <si>
+    <t>Walk trials C1-C3 (files)</t>
   </si>
 </sst>
 </file>
@@ -1040,7 +1046,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:K51"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
@@ -1052,10 +1058,11 @@
     <col min="9" max="9" width="24.33203125" customWidth="1"/>
     <col min="10" max="10" width="19.33203125" customWidth="1"/>
     <col min="11" max="11" width="19.77734375" customWidth="1"/>
+    <col min="14" max="14" width="16.6640625" customWidth="1"/>
     <col min="15" max="15" width="8.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1075,7 +1082,7 @@
         <v>62</v>
       </c>
       <c r="H1" t="s">
-        <v>63</v>
+        <v>91</v>
       </c>
       <c r="I1" t="s">
         <v>64</v>
@@ -1086,8 +1093,11 @@
       <c r="K1" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="2" spans="1:11">
+      <c r="N1" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1107,10 +1117,13 @@
         <v>1</v>
       </c>
       <c r="H2">
+        <v>15</v>
+      </c>
+      <c r="N2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:14">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1130,10 +1143,13 @@
         <v>1</v>
       </c>
       <c r="H3">
+        <v>11</v>
+      </c>
+      <c r="N3">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:14">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1153,10 +1169,13 @@
         <v>1</v>
       </c>
       <c r="H4">
+        <v>13</v>
+      </c>
+      <c r="N4">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:14">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1176,10 +1195,13 @@
         <v>1</v>
       </c>
       <c r="H5">
+        <v>14</v>
+      </c>
+      <c r="N5">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:14">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1199,10 +1221,13 @@
         <v>0</v>
       </c>
       <c r="H6">
+        <v>15</v>
+      </c>
+      <c r="N6">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:14">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1222,10 +1247,13 @@
         <v>1</v>
       </c>
       <c r="H7">
+        <v>13</v>
+      </c>
+      <c r="N7">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:14">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1245,10 +1273,13 @@
         <v>1</v>
       </c>
       <c r="H8">
+        <v>14</v>
+      </c>
+      <c r="N8">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:14">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1268,10 +1299,13 @@
         <v>0</v>
       </c>
       <c r="H9">
+        <v>15</v>
+      </c>
+      <c r="N9">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:14">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1291,10 +1325,13 @@
         <v>0</v>
       </c>
       <c r="H10">
+        <v>15</v>
+      </c>
+      <c r="N10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:14">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1314,10 +1351,13 @@
         <v>1</v>
       </c>
       <c r="H11">
+        <v>13</v>
+      </c>
+      <c r="N11">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:14">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1337,10 +1377,13 @@
         <v>1</v>
       </c>
       <c r="H12">
+        <v>13</v>
+      </c>
+      <c r="N12">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:14">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1360,10 +1403,13 @@
         <v>1</v>
       </c>
       <c r="H13">
+        <v>14</v>
+      </c>
+      <c r="N13">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:14">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1383,10 +1429,13 @@
         <v>0</v>
       </c>
       <c r="H14">
+        <v>15</v>
+      </c>
+      <c r="N14">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:14">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1406,10 +1455,13 @@
         <v>1</v>
       </c>
       <c r="H15">
+        <v>12</v>
+      </c>
+      <c r="N15">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:14">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1429,10 +1481,13 @@
         <v>1</v>
       </c>
       <c r="H16">
+        <v>15</v>
+      </c>
+      <c r="N16">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:14">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1452,10 +1507,13 @@
         <v>1</v>
       </c>
       <c r="H17">
+        <v>14</v>
+      </c>
+      <c r="N17">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:14">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1475,10 +1533,13 @@
         <v>1</v>
       </c>
       <c r="H18">
+        <v>15</v>
+      </c>
+      <c r="N18">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:14">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1498,10 +1559,13 @@
         <v>1</v>
       </c>
       <c r="H19">
+        <v>15</v>
+      </c>
+      <c r="N19">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:14">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1521,10 +1585,13 @@
         <v>1</v>
       </c>
       <c r="H20">
+        <v>15</v>
+      </c>
+      <c r="N20">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:14">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1544,10 +1611,13 @@
         <v>1</v>
       </c>
       <c r="H21">
+        <v>13</v>
+      </c>
+      <c r="N21">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:14">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1567,10 +1637,13 @@
         <v>1</v>
       </c>
       <c r="H22">
+        <v>13</v>
+      </c>
+      <c r="N22">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:14">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1590,10 +1663,13 @@
         <v>1</v>
       </c>
       <c r="H23">
+        <v>11</v>
+      </c>
+      <c r="N23">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:14">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1613,10 +1689,13 @@
         <v>1</v>
       </c>
       <c r="H24">
+        <v>13</v>
+      </c>
+      <c r="N24">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:14">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1636,10 +1715,13 @@
         <v>0</v>
       </c>
       <c r="H25">
+        <v>15</v>
+      </c>
+      <c r="N25">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:14">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1659,10 +1741,13 @@
         <v>1</v>
       </c>
       <c r="H26">
+        <v>14</v>
+      </c>
+      <c r="N26">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:14">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1682,10 +1767,13 @@
         <v>0</v>
       </c>
       <c r="H27">
+        <v>15</v>
+      </c>
+      <c r="N27">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:14">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1705,10 +1793,13 @@
         <v>0</v>
       </c>
       <c r="H28">
+        <v>15</v>
+      </c>
+      <c r="N28">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:14">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1728,10 +1819,13 @@
         <v>1</v>
       </c>
       <c r="H29">
+        <v>15</v>
+      </c>
+      <c r="N29">
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:14">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1751,10 +1845,13 @@
         <v>1</v>
       </c>
       <c r="H30">
+        <v>13</v>
+      </c>
+      <c r="N30">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:14">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1774,10 +1871,13 @@
         <v>1</v>
       </c>
       <c r="H31">
+        <v>11</v>
+      </c>
+      <c r="N31">
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:14">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1794,13 +1894,16 @@
         <v>1.74</v>
       </c>
       <c r="G32">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H32">
+        <v>15</v>
+      </c>
+      <c r="N32">
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:14">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1820,10 +1923,13 @@
         <v>0</v>
       </c>
       <c r="H33">
+        <v>15</v>
+      </c>
+      <c r="N33">
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:14">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1840,13 +1946,16 @@
         <v>1.7</v>
       </c>
       <c r="G34">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H34">
+        <v>15</v>
+      </c>
+      <c r="N34">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:14">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1866,10 +1975,13 @@
         <v>1</v>
       </c>
       <c r="H35">
+        <v>15</v>
+      </c>
+      <c r="N35">
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:14">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1889,10 +2001,13 @@
         <v>1</v>
       </c>
       <c r="H36">
+        <v>15</v>
+      </c>
+      <c r="N36">
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:14">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1912,10 +2027,13 @@
         <v>1</v>
       </c>
       <c r="H37">
+        <v>14</v>
+      </c>
+      <c r="N37">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:14">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1935,10 +2053,13 @@
         <v>0</v>
       </c>
       <c r="H38">
+        <v>15</v>
+      </c>
+      <c r="N38">
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:14">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1958,10 +2079,13 @@
         <v>1</v>
       </c>
       <c r="H39">
+        <v>12</v>
+      </c>
+      <c r="N39">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:14">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1981,10 +2105,13 @@
         <v>1</v>
       </c>
       <c r="H40">
+        <v>15</v>
+      </c>
+      <c r="N40">
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:14">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2004,10 +2131,13 @@
         <v>1</v>
       </c>
       <c r="H41">
+        <v>15</v>
+      </c>
+      <c r="N41">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:14">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2027,10 +2157,13 @@
         <v>1</v>
       </c>
       <c r="H42">
+        <v>14</v>
+      </c>
+      <c r="N42">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:14">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2050,10 +2183,13 @@
         <v>1</v>
       </c>
       <c r="H43">
+        <v>13</v>
+      </c>
+      <c r="N43">
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:14">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2073,10 +2209,13 @@
         <v>1</v>
       </c>
       <c r="H44">
+        <v>14</v>
+      </c>
+      <c r="N44">
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:14">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2096,10 +2235,13 @@
         <v>1</v>
       </c>
       <c r="H45">
+        <v>13</v>
+      </c>
+      <c r="N45">
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:14">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2119,10 +2261,13 @@
         <v>1</v>
       </c>
       <c r="H46">
+        <v>13</v>
+      </c>
+      <c r="N46">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:14">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2142,10 +2287,13 @@
         <v>1</v>
       </c>
       <c r="H47">
+        <v>14</v>
+      </c>
+      <c r="N47">
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:14">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2165,10 +2313,13 @@
         <v>1</v>
       </c>
       <c r="H48">
+        <v>13</v>
+      </c>
+      <c r="N48">
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:14">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2188,10 +2339,13 @@
         <v>1</v>
       </c>
       <c r="H49">
+        <v>13</v>
+      </c>
+      <c r="N49">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:14">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2211,10 +2365,13 @@
         <v>1</v>
       </c>
       <c r="H50">
+        <v>14</v>
+      </c>
+      <c r="N50">
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:14">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2234,6 +2391,9 @@
         <v>0</v>
       </c>
       <c r="H51">
+        <v>15</v>
+      </c>
+      <c r="N51">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added columns to report excluded data
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A1DEBBE-F192-4550-9A6E-2862CEA70DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD54C56-D4C2-4FF0-B3D0-0A3DD8804CC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="93">
   <si>
     <t>Database No.</t>
   </si>
@@ -250,16 +250,7 @@
     <t>Calib pose</t>
   </si>
   <si>
-    <t>Walk trials (files)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Usable trials </t>
-  </si>
-  <si>
-    <t>Duration per trials (s)</t>
-  </si>
-  <si>
-    <t>Wrong trials (reason)</t>
   </si>
   <si>
     <t>M</t>
@@ -353,6 +344,18 @@
   </si>
   <si>
     <t>0–0.4 m.s−1 (C1), 0.4–0.8 m.s−1 (C2), 0.8–1.2 m.s−1 (C3). Self-selected spontaneous (C4) and fast (C5)</t>
+  </si>
+  <si>
+    <t>Wrong trials - processing (reason)</t>
+  </si>
+  <si>
+    <t>Wrong trials - visual inspection (reason)</t>
+  </si>
+  <si>
+    <t>Excluded trials (reason: speed / step-width)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Walk trials </t>
   </si>
 </sst>
 </file>
@@ -742,19 +745,19 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C2">
         <v>2019</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E2" t="s">
         <v>19</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="G2">
         <v>50</v>
@@ -766,28 +769,28 @@
         <v>26</v>
       </c>
       <c r="J2" t="s">
+        <v>76</v>
+      </c>
+      <c r="K2" t="s">
+        <v>77</v>
+      </c>
+      <c r="L2" t="s">
+        <v>78</v>
+      </c>
+      <c r="M2" t="s">
+        <v>80</v>
+      </c>
+      <c r="N2" t="s">
         <v>79</v>
       </c>
-      <c r="K2" t="s">
-        <v>80</v>
-      </c>
-      <c r="L2" t="s">
+      <c r="O2" t="s">
         <v>81</v>
-      </c>
-      <c r="M2" t="s">
-        <v>83</v>
-      </c>
-      <c r="N2" t="s">
-        <v>82</v>
-      </c>
-      <c r="O2" t="s">
-        <v>84</v>
       </c>
       <c r="P2">
         <v>2</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:18" ht="43.2">
@@ -807,7 +810,7 @@
         <v>19</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="G3">
         <v>13</v>
@@ -851,7 +854,7 @@
         <v>19</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="G4" s="1">
         <v>10</v>
@@ -1055,23 +1058,26 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:N52"/>
+  <dimension ref="A1:P52"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="10.21875" customWidth="1"/>
     <col min="2" max="2" width="10.77734375" customWidth="1"/>
     <col min="3" max="3" width="10.44140625" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="5" max="6" width="12" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="5.33203125" customWidth="1"/>
+    <col min="7" max="7" width="11.88671875" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="24.33203125" customWidth="1"/>
-    <col min="10" max="10" width="19.33203125" customWidth="1"/>
-    <col min="11" max="11" width="19.77734375" customWidth="1"/>
-    <col min="14" max="14" width="16.6640625" customWidth="1"/>
-    <col min="15" max="15" width="8.77734375" customWidth="1"/>
+    <col min="9" max="9" width="29.33203125" customWidth="1"/>
+    <col min="10" max="10" width="34.44140625" customWidth="1"/>
+    <col min="11" max="11" width="37.109375" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" customWidth="1"/>
+    <col min="13" max="13" width="8.77734375" customWidth="1"/>
+    <col min="16" max="16" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:16">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -1091,22 +1097,25 @@
         <v>62</v>
       </c>
       <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
         <v>90</v>
       </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
       <c r="K1" t="s">
-        <v>66</v>
-      </c>
-      <c r="N1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1114,7 +1123,7 @@
         <v>31</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D2">
         <v>67</v>
@@ -1128,11 +1137,11 @@
       <c r="H2">
         <v>15</v>
       </c>
-      <c r="N2">
+      <c r="P2">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:16">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1140,7 +1149,7 @@
         <v>48</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D3">
         <v>65.400000000000006</v>
@@ -1154,11 +1163,11 @@
       <c r="H3">
         <v>11</v>
       </c>
-      <c r="N3">
+      <c r="P3">
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:16">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1166,7 +1175,7 @@
         <v>28</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D4">
         <v>50</v>
@@ -1180,11 +1189,11 @@
       <c r="H4">
         <v>13</v>
       </c>
-      <c r="N4">
+      <c r="P4">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:16">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1192,7 +1201,7 @@
         <v>23</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5">
         <v>72.5</v>
@@ -1206,11 +1215,11 @@
       <c r="H5">
         <v>14</v>
       </c>
-      <c r="N5">
+      <c r="P5">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:16">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1218,7 +1227,7 @@
         <v>25</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D6">
         <v>73.5</v>
@@ -1232,11 +1241,11 @@
       <c r="H6">
         <v>15</v>
       </c>
-      <c r="N6">
+      <c r="P6">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:16">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1244,7 +1253,7 @@
         <v>23</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D7">
         <v>73</v>
@@ -1258,11 +1267,11 @@
       <c r="H7">
         <v>13</v>
       </c>
-      <c r="N7">
+      <c r="P7">
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:16">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1270,7 +1279,7 @@
         <v>44</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D8">
         <v>65</v>
@@ -1284,11 +1293,11 @@
       <c r="H8">
         <v>14</v>
       </c>
-      <c r="N8">
+      <c r="P8">
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:16">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1296,7 +1305,7 @@
         <v>30</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D9">
         <v>57.1</v>
@@ -1310,11 +1319,11 @@
       <c r="H9">
         <v>15</v>
       </c>
-      <c r="N9">
+      <c r="P9">
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:16">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1322,7 +1331,7 @@
         <v>57</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D10">
         <v>86</v>
@@ -1336,11 +1345,11 @@
       <c r="H10">
         <v>15</v>
       </c>
-      <c r="N10">
+      <c r="P10">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:16">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1348,7 +1357,7 @@
         <v>59</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D11">
         <v>63.4</v>
@@ -1362,11 +1371,11 @@
       <c r="H11">
         <v>13</v>
       </c>
-      <c r="N11">
+      <c r="P11">
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:16">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1374,7 +1383,7 @@
         <v>26</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D12">
         <v>61.3</v>
@@ -1388,11 +1397,11 @@
       <c r="H12">
         <v>13</v>
       </c>
-      <c r="N12">
+      <c r="P12">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:16">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1400,7 +1409,7 @@
         <v>29</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D13">
         <v>92</v>
@@ -1414,11 +1423,11 @@
       <c r="H13">
         <v>14</v>
       </c>
-      <c r="N13">
+      <c r="P13">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:16">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1426,7 +1435,7 @@
         <v>22</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D14">
         <v>67</v>
@@ -1440,11 +1449,11 @@
       <c r="H14">
         <v>15</v>
       </c>
-      <c r="N14">
+      <c r="P14">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:16">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1452,7 +1461,7 @@
         <v>26</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D15">
         <v>73.8</v>
@@ -1466,11 +1475,11 @@
       <c r="H15">
         <v>12</v>
       </c>
-      <c r="N15">
+      <c r="P15">
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:16">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1478,7 +1487,7 @@
         <v>48</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D16">
         <v>59.8</v>
@@ -1492,11 +1501,11 @@
       <c r="H16">
         <v>15</v>
       </c>
-      <c r="N16">
+      <c r="P16">
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:16">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1504,7 +1513,7 @@
         <v>33</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D17">
         <v>87.5</v>
@@ -1518,11 +1527,11 @@
       <c r="H17">
         <v>14</v>
       </c>
-      <c r="N17">
+      <c r="P17">
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:16">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1530,7 +1539,7 @@
         <v>31</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D18">
         <v>80.5</v>
@@ -1544,11 +1553,11 @@
       <c r="H18">
         <v>15</v>
       </c>
-      <c r="N18">
+      <c r="P18">
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:16">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1556,7 +1565,7 @@
         <v>38</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D19">
         <v>89.9</v>
@@ -1570,11 +1579,11 @@
       <c r="H19">
         <v>15</v>
       </c>
-      <c r="N19">
+      <c r="P19">
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:16">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1582,7 +1591,7 @@
         <v>62</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D20">
         <v>60.7</v>
@@ -1596,11 +1605,11 @@
       <c r="H20">
         <v>15</v>
       </c>
-      <c r="N20">
+      <c r="P20">
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:16">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1608,7 +1617,7 @@
         <v>21</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D21">
         <v>67.2</v>
@@ -1622,11 +1631,11 @@
       <c r="H21">
         <v>13</v>
       </c>
-      <c r="N21">
+      <c r="P21">
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:16">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1634,7 +1643,7 @@
         <v>24</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D22">
         <v>63.5</v>
@@ -1648,11 +1657,11 @@
       <c r="H22">
         <v>13</v>
       </c>
-      <c r="N22">
+      <c r="P22">
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:16">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1660,7 +1669,7 @@
         <v>21</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D23">
         <v>89.6</v>
@@ -1674,11 +1683,11 @@
       <c r="H23">
         <v>11</v>
       </c>
-      <c r="N23">
+      <c r="P23">
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:16">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1686,7 +1695,7 @@
         <v>19</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D24">
         <v>56.5</v>
@@ -1700,11 +1709,11 @@
       <c r="H24">
         <v>13</v>
       </c>
-      <c r="N24">
+      <c r="P24">
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:16">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1712,7 +1721,7 @@
         <v>40</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D25">
         <v>61.8</v>
@@ -1726,11 +1735,11 @@
       <c r="H25">
         <v>15</v>
       </c>
-      <c r="N25">
+      <c r="P25">
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:16">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1738,7 +1747,7 @@
         <v>40</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D26">
         <v>61.5</v>
@@ -1752,11 +1761,11 @@
       <c r="H26">
         <v>14</v>
       </c>
-      <c r="N26">
+      <c r="P26">
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:16">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1764,7 +1773,7 @@
         <v>32</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D27">
         <v>72.2</v>
@@ -1778,11 +1787,11 @@
       <c r="H27">
         <v>15</v>
       </c>
-      <c r="N27">
+      <c r="P27">
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:16">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1790,7 +1799,7 @@
         <v>28</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D28">
         <v>61.9</v>
@@ -1804,11 +1813,11 @@
       <c r="H28">
         <v>15</v>
       </c>
-      <c r="N28">
+      <c r="P28">
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:16">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1816,7 +1825,7 @@
         <v>25</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D29">
         <v>88</v>
@@ -1830,11 +1839,11 @@
       <c r="H29">
         <v>15</v>
       </c>
-      <c r="N29">
+      <c r="P29">
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:16">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1842,7 +1851,7 @@
         <v>25</v>
       </c>
       <c r="C30" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D30">
         <v>79.5</v>
@@ -1856,11 +1865,11 @@
       <c r="H30">
         <v>13</v>
       </c>
-      <c r="N30">
+      <c r="P30">
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:16">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1868,7 +1877,7 @@
         <v>21</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D31">
         <v>62.8</v>
@@ -1882,11 +1891,11 @@
       <c r="H31">
         <v>11</v>
       </c>
-      <c r="N31">
+      <c r="P31">
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:16">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1894,7 +1903,7 @@
         <v>39</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D32">
         <v>74</v>
@@ -1908,11 +1917,11 @@
       <c r="H32">
         <v>15</v>
       </c>
-      <c r="N32">
+      <c r="P32">
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:16">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1920,7 +1929,7 @@
         <v>52</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D33">
         <v>87.2</v>
@@ -1934,11 +1943,11 @@
       <c r="H33">
         <v>15</v>
       </c>
-      <c r="N33">
+      <c r="P33">
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:16">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1946,7 +1955,7 @@
         <v>35</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D34">
         <v>62</v>
@@ -1960,11 +1969,11 @@
       <c r="H34">
         <v>15</v>
       </c>
-      <c r="N34">
+      <c r="P34">
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:16">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1972,7 +1981,7 @@
         <v>48</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D35">
         <v>89.4</v>
@@ -1986,11 +1995,11 @@
       <c r="H35">
         <v>15</v>
       </c>
-      <c r="N35">
+      <c r="P35">
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:14">
+    <row r="36" spans="1:16">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1998,7 +2007,7 @@
         <v>63</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D36">
         <v>60.2</v>
@@ -2012,11 +2021,11 @@
       <c r="H36">
         <v>15</v>
       </c>
-      <c r="N36">
+      <c r="P36">
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:14">
+    <row r="37" spans="1:16">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2024,7 +2033,7 @@
         <v>58</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D37">
         <v>73</v>
@@ -2038,11 +2047,11 @@
       <c r="H37">
         <v>14</v>
       </c>
-      <c r="N37">
+      <c r="P37">
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:14">
+    <row r="38" spans="1:16">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2050,7 +2059,7 @@
         <v>50</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D38">
         <v>68</v>
@@ -2064,11 +2073,11 @@
       <c r="H38">
         <v>15</v>
       </c>
-      <c r="N38">
+      <c r="P38">
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:14">
+    <row r="39" spans="1:16">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2076,7 +2085,7 @@
         <v>46</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D39">
         <v>76</v>
@@ -2090,11 +2099,11 @@
       <c r="H39">
         <v>12</v>
       </c>
-      <c r="N39">
+      <c r="P39">
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:14">
+    <row r="40" spans="1:16">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2102,7 +2111,7 @@
         <v>41</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D40">
         <v>60.5</v>
@@ -2116,11 +2125,11 @@
       <c r="H40">
         <v>15</v>
       </c>
-      <c r="N40">
+      <c r="P40">
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:14">
+    <row r="41" spans="1:16">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2128,7 +2137,7 @@
         <v>43</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D41">
         <v>95</v>
@@ -2142,11 +2151,11 @@
       <c r="H41">
         <v>15</v>
       </c>
-      <c r="N41">
+      <c r="P41">
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:14">
+    <row r="42" spans="1:16">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2154,7 +2163,7 @@
         <v>30</v>
       </c>
       <c r="C42" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D42">
         <v>58</v>
@@ -2168,11 +2177,11 @@
       <c r="H42">
         <v>14</v>
       </c>
-      <c r="N42">
+      <c r="P42">
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:14">
+    <row r="43" spans="1:16">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2180,7 +2189,7 @@
         <v>64</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D43">
         <v>51.5</v>
@@ -2194,11 +2203,11 @@
       <c r="H43">
         <v>13</v>
       </c>
-      <c r="N43">
+      <c r="P43">
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:14">
+    <row r="44" spans="1:16">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2206,7 +2215,7 @@
         <v>51</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D44">
         <v>65.5</v>
@@ -2220,11 +2229,11 @@
       <c r="H44">
         <v>14</v>
       </c>
-      <c r="N44">
+      <c r="P44">
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:14">
+    <row r="45" spans="1:16">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2232,7 +2241,7 @@
         <v>24</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D45">
         <v>86</v>
@@ -2246,11 +2255,11 @@
       <c r="H45">
         <v>13</v>
       </c>
-      <c r="N45">
+      <c r="P45">
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:14">
+    <row r="46" spans="1:16">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2258,7 +2267,7 @@
         <v>26</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D46">
         <v>50.8</v>
@@ -2272,11 +2281,11 @@
       <c r="H46">
         <v>13</v>
       </c>
-      <c r="N46">
+      <c r="P46">
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:14">
+    <row r="47" spans="1:16">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2284,7 +2293,7 @@
         <v>38</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D47">
         <v>81.5</v>
@@ -2298,11 +2307,11 @@
       <c r="H47">
         <v>14</v>
       </c>
-      <c r="N47">
+      <c r="P47">
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:14">
+    <row r="48" spans="1:16">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2310,7 +2319,7 @@
         <v>42</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D48">
         <v>66.099999999999994</v>
@@ -2324,11 +2333,11 @@
       <c r="H48">
         <v>13</v>
       </c>
-      <c r="N48">
+      <c r="P48">
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:14">
+    <row r="49" spans="1:16">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2336,7 +2345,7 @@
         <v>31</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D49">
         <v>74.8</v>
@@ -2350,11 +2359,11 @@
       <c r="H49">
         <v>13</v>
       </c>
-      <c r="N49">
+      <c r="P49">
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:14">
+    <row r="50" spans="1:16">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2362,7 +2371,7 @@
         <v>67</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D50">
         <v>98</v>
@@ -2376,11 +2385,11 @@
       <c r="H50">
         <v>14</v>
       </c>
-      <c r="N50">
+      <c r="P50">
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:14">
+    <row r="51" spans="1:16">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2388,7 +2397,7 @@
         <v>21</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D51">
         <v>74</v>
@@ -2402,11 +2411,11 @@
       <c r="H51">
         <v>15</v>
       </c>
-      <c r="N51">
+      <c r="P51">
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:14">
+    <row r="52" spans="1:16">
       <c r="H52" s="8">
         <f>SUM(H2:H51)</f>
         <v>696</v>
@@ -2420,15 +2429,18 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="9" max="9" width="14.109375" customWidth="1"/>
-    <col min="10" max="10" width="19.109375" customWidth="1"/>
-    <col min="11" max="11" width="28.33203125" customWidth="1"/>
+    <col min="8" max="8" width="10.44140625" customWidth="1"/>
+    <col min="9" max="9" width="30.6640625" customWidth="1"/>
+    <col min="10" max="10" width="33.21875" customWidth="1"/>
+    <col min="11" max="11" width="36.6640625" customWidth="1"/>
+    <col min="12" max="12" width="15.44140625" customWidth="1"/>
+    <col min="14" max="14" width="14.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -2448,19 +2460,22 @@
         <v>62</v>
       </c>
       <c r="H1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
         <v>63</v>
       </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2468,7 +2483,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D2">
         <v>74</v>
@@ -2482,14 +2497,14 @@
       <c r="H2">
         <v>21</v>
       </c>
-      <c r="I2">
+      <c r="J2" t="s">
+        <v>85</v>
+      </c>
+      <c r="L2">
         <v>17</v>
       </c>
-      <c r="K2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2497,7 +2512,7 @@
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D3">
         <v>72</v>
@@ -2511,14 +2526,14 @@
       <c r="H3">
         <v>23</v>
       </c>
-      <c r="I3">
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="L3">
         <v>23</v>
       </c>
-      <c r="K3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2526,7 +2541,7 @@
         <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D4">
         <v>80</v>
@@ -2540,14 +2555,14 @@
       <c r="H4">
         <v>24</v>
       </c>
-      <c r="I4">
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="L4">
         <v>24</v>
       </c>
-      <c r="K4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2555,7 +2570,7 @@
         <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5">
         <v>60</v>
@@ -2569,11 +2584,11 @@
       <c r="H5">
         <v>17</v>
       </c>
-      <c r="K5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11">
+      <c r="J5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2581,7 +2596,7 @@
         <v>21</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D6">
         <v>71</v>
@@ -2596,7 +2611,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2604,7 +2619,7 @@
         <v>20</v>
       </c>
       <c r="C7" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D7">
         <v>65</v>
@@ -2619,7 +2634,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8">
         <v>7</v>
       </c>
@@ -2627,7 +2642,7 @@
         <v>25</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D8">
         <v>72</v>
@@ -2642,7 +2657,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2650,7 +2665,7 @@
         <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D9">
         <v>85</v>
@@ -2665,7 +2680,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2673,7 +2688,7 @@
         <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D10">
         <v>76</v>
@@ -2688,7 +2703,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11">
         <v>10</v>
       </c>
@@ -2696,7 +2711,7 @@
         <v>20</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D11">
         <v>80</v>
@@ -2710,11 +2725,11 @@
       <c r="H11">
         <v>23</v>
       </c>
-      <c r="K11">
+      <c r="J11">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2722,7 +2737,7 @@
         <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D12">
         <v>75</v>
@@ -2736,11 +2751,11 @@
       <c r="H12">
         <v>27</v>
       </c>
-      <c r="K12" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11">
+      <c r="J12" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13">
         <v>12</v>
       </c>
@@ -2748,7 +2763,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D13">
         <v>80</v>
@@ -2763,7 +2778,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:12">
       <c r="A14">
         <v>13</v>
       </c>
@@ -2771,7 +2786,7 @@
         <v>21</v>
       </c>
       <c r="C14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D14">
         <v>58</v>
@@ -2786,7 +2801,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:12">
       <c r="H15" s="8">
         <f>SUM(H1:H14)</f>
         <v>302</v>
@@ -2800,13 +2815,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="11" max="11" width="19.109375" customWidth="1"/>
+    <col min="8" max="8" width="10.88671875" customWidth="1"/>
+    <col min="9" max="9" width="28.88671875" customWidth="1"/>
+    <col min="10" max="10" width="33.21875" customWidth="1"/>
+    <col min="11" max="11" width="36.6640625" customWidth="1"/>
+    <col min="12" max="12" width="13.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -2826,33 +2845,36 @@
         <v>62</v>
       </c>
       <c r="H1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
         <v>63</v>
       </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -2861,21 +2883,21 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -2884,21 +2906,21 @@
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:12">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -2907,21 +2929,21 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:12">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G5">
         <v>0</v>
@@ -2930,21 +2952,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -2953,21 +2975,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -2976,21 +2998,21 @@
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -2999,21 +3021,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G9">
         <v>0</v>
@@ -3022,21 +3044,21 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:12">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -3045,21 +3067,21 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:12">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -3068,13 +3090,13 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:12">
       <c r="H12" s="8">
         <f>SUM(H2:H11)</f>
         <v>167</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:12">
       <c r="H13" s="8"/>
     </row>
   </sheetData>
@@ -3085,13 +3107,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
-    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="8" max="8" width="11.5546875" customWidth="1"/>
+    <col min="9" max="9" width="29.77734375" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="11" max="11" width="36.77734375" customWidth="1"/>
+    <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>57</v>
       </c>
@@ -3111,27 +3137,30 @@
         <v>62</v>
       </c>
       <c r="H1" t="s">
+        <v>92</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
         <v>63</v>
       </c>
-      <c r="I1" t="s">
-        <v>64</v>
-      </c>
-      <c r="J1" t="s">
-        <v>65</v>
-      </c>
-      <c r="K1" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11">
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C2" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D2">
         <v>69.86</v>
@@ -3142,22 +3171,22 @@
       <c r="H2">
         <v>3</v>
       </c>
-      <c r="I2">
+      <c r="I2" t="s">
+        <v>69</v>
+      </c>
+      <c r="L2">
         <v>0</v>
       </c>
-      <c r="K2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D3">
         <v>66.680000000000007</v>
@@ -3168,22 +3197,22 @@
       <c r="H3">
         <v>4</v>
       </c>
-      <c r="I3">
+      <c r="I3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L3">
         <v>3</v>
       </c>
-      <c r="K3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D4">
         <v>53.07</v>
@@ -3194,19 +3223,19 @@
       <c r="H4">
         <v>3</v>
       </c>
-      <c r="K4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
+      <c r="I4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D5">
         <v>71.67</v>
@@ -3218,15 +3247,15 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:12">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D6">
         <v>90.7</v>
@@ -3238,15 +3267,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:12">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D7">
         <v>48.99</v>
@@ -3258,15 +3287,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:12">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C8" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D8">
         <v>63.96</v>
@@ -3278,7 +3307,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:12">
       <c r="H9" s="8">
         <f>SUM(H1:H8)</f>
         <v>18</v>

</xml_diff>

<commit_message>
Update DB Simonlehner to DB3
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C030D6DE-5098-41C9-B831-0E035D95FD20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49931A1C-06FC-4BCE-92DB-2F6EA8A12911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="DB1" sheetId="2" r:id="rId2"/>
     <sheet name="DB2" sheetId="3" r:id="rId3"/>
-    <sheet name="DB3" sheetId="4" r:id="rId4"/>
-    <sheet name="DB4" sheetId="5" r:id="rId5"/>
+    <sheet name="DB3" sheetId="6" r:id="rId4"/>
+    <sheet name="DB4" sheetId="7" r:id="rId5"/>
+    <sheet name="DB Grouvel" sheetId="4" r:id="rId6"/>
+    <sheet name="DB Han" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="94">
   <si>
     <t>Database No.</t>
   </si>
@@ -356,6 +358,9 @@
   </si>
   <si>
     <t xml:space="preserve">Walk trials </t>
+  </si>
+  <si>
+    <t>Simonlehner</t>
   </si>
 </sst>
 </file>
@@ -430,12 +435,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -452,7 +463,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -470,6 +481,7 @@
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -665,7 +677,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R11"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="11.77734375" customWidth="1"/>
@@ -837,95 +849,17 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="46.8">
-      <c r="A4">
+    <row r="4" spans="1:18">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C4">
-        <v>2023</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="G4" s="1">
-        <v>10</v>
-      </c>
-      <c r="H4" s="1">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" s="9">
         <v>4</v>
-      </c>
-      <c r="I4" s="1">
-        <v>6</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="R4" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" ht="43.2">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5">
-        <v>2023</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="G5" s="1">
-        <v>7</v>
-      </c>
-      <c r="H5" s="1">
-        <v>4</v>
-      </c>
-      <c r="I5" s="1">
-        <v>3</v>
-      </c>
-      <c r="J5" t="s">
-        <v>35</v>
-      </c>
-      <c r="K5" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" t="s">
-        <v>37</v>
-      </c>
-      <c r="O5" s="1">
-        <v>96</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="R5" s="1" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" spans="1:18">
@@ -1040,12 +974,97 @@
         <v>56</v>
       </c>
     </row>
+    <row r="12" spans="1:18" ht="46.8">
+      <c r="B12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12">
+        <v>2023</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G12" s="1">
+        <v>10</v>
+      </c>
+      <c r="H12" s="1">
+        <v>4</v>
+      </c>
+      <c r="I12" s="1">
+        <v>6</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="R12" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" ht="43.2">
+      <c r="B13" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C13">
+        <v>2023</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G13" s="1">
+        <v>7</v>
+      </c>
+      <c r="H13" s="1">
+        <v>4</v>
+      </c>
+      <c r="I13" s="1">
+        <v>3</v>
+      </c>
+      <c r="J13" t="s">
+        <v>35</v>
+      </c>
+      <c r="K13" t="s">
+        <v>36</v>
+      </c>
+      <c r="L13" t="s">
+        <v>37</v>
+      </c>
+      <c r="O13" s="1">
+        <v>96</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="R3" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="R4" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="Q5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="R5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="R12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="Q13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="R13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="R9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="R10" r:id="rId6" location="Bib1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
     <hyperlink ref="R11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
@@ -2844,6 +2863,102 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3518C62A-2ABA-4532-ADB0-E26CA60F7C0C}">
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5634500B-8BBC-4D8B-92B7-7498A6AEDFBA}">
+  <dimension ref="A1:P1"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:16">
+      <c r="A1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" t="s">
+        <v>62</v>
+      </c>
+      <c r="H1" t="s">
+        <v>87</v>
+      </c>
+      <c r="I1" t="s">
+        <v>89</v>
+      </c>
+      <c r="J1" t="s">
+        <v>90</v>
+      </c>
+      <c r="K1" t="s">
+        <v>91</v>
+      </c>
+      <c r="L1" t="s">
+        <v>63</v>
+      </c>
+      <c r="P1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:L13"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
@@ -3141,7 +3256,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>

</xml_diff>

<commit_message>
Update DB1 usable trials
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49931A1C-06FC-4BCE-92DB-2F6EA8A12911}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3450F48-C74F-480D-9B75-F88F06CADCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -1088,9 +1088,9 @@
     <col min="6" max="6" width="5.33203125" customWidth="1"/>
     <col min="7" max="7" width="11.88671875" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" customWidth="1"/>
-    <col min="9" max="9" width="29.33203125" customWidth="1"/>
-    <col min="10" max="10" width="34.44140625" customWidth="1"/>
-    <col min="11" max="11" width="37.109375" customWidth="1"/>
+    <col min="9" max="9" width="17" customWidth="1"/>
+    <col min="10" max="10" width="16.77734375" customWidth="1"/>
+    <col min="11" max="11" width="13" customWidth="1"/>
     <col min="12" max="12" width="9.33203125" customWidth="1"/>
     <col min="13" max="13" width="8.77734375" customWidth="1"/>
     <col min="16" max="16" width="16.6640625" customWidth="1"/>
@@ -1157,7 +1157,7 @@
         <v>15</v>
       </c>
       <c r="L2">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P2">
         <v>10</v>
@@ -1244,7 +1244,7 @@
         <v>14</v>
       </c>
       <c r="L5">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="P5">
         <v>9</v>

</xml_diff>

<commit_message>
DB1 P01-P10 Usable trials
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3450F48-C74F-480D-9B75-F88F06CADCA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56767C10-220C-4409-9C20-B0CC92373D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="95">
   <si>
     <t>Database No.</t>
   </si>
@@ -361,6 +361,9 @@
   </si>
   <si>
     <t>Simonlehner</t>
+  </si>
+  <si>
+    <t>"ID not run" for the others</t>
   </si>
 </sst>
 </file>
@@ -1156,6 +1159,9 @@
       <c r="H2">
         <v>15</v>
       </c>
+      <c r="I2" t="s">
+        <v>94</v>
+      </c>
       <c r="L2">
         <v>8</v>
       </c>
@@ -1185,6 +1191,9 @@
       <c r="H3">
         <v>11</v>
       </c>
+      <c r="I3" t="s">
+        <v>94</v>
+      </c>
       <c r="L3">
         <v>4</v>
       </c>
@@ -1214,6 +1223,9 @@
       <c r="H4">
         <v>13</v>
       </c>
+      <c r="I4" t="s">
+        <v>94</v>
+      </c>
       <c r="L4">
         <v>1</v>
       </c>
@@ -1243,6 +1255,9 @@
       <c r="H5">
         <v>14</v>
       </c>
+      <c r="I5" t="s">
+        <v>94</v>
+      </c>
       <c r="L5">
         <v>6</v>
       </c>
@@ -1272,6 +1287,9 @@
       <c r="H6">
         <v>15</v>
       </c>
+      <c r="I6" t="s">
+        <v>94</v>
+      </c>
       <c r="L6">
         <v>6</v>
       </c>
@@ -1301,6 +1319,9 @@
       <c r="H7">
         <v>13</v>
       </c>
+      <c r="I7" t="s">
+        <v>94</v>
+      </c>
       <c r="L7">
         <v>8</v>
       </c>
@@ -1330,6 +1351,9 @@
       <c r="H8">
         <v>14</v>
       </c>
+      <c r="I8" t="s">
+        <v>94</v>
+      </c>
       <c r="L8">
         <v>4</v>
       </c>
@@ -1359,6 +1383,9 @@
       <c r="H9">
         <v>15</v>
       </c>
+      <c r="I9" t="s">
+        <v>94</v>
+      </c>
       <c r="L9">
         <v>9</v>
       </c>
@@ -1388,6 +1415,9 @@
       <c r="H10">
         <v>15</v>
       </c>
+      <c r="I10" t="s">
+        <v>94</v>
+      </c>
       <c r="L10">
         <v>9</v>
       </c>
@@ -1416,6 +1446,9 @@
       </c>
       <c r="H11">
         <v>13</v>
+      </c>
+      <c r="I11" t="s">
+        <v>94</v>
       </c>
       <c r="L11">
         <v>4</v>

</xml_diff>

<commit_message>
Update DB3 P04-P08 info
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56767C10-220C-4409-9C20-B0CC92373D1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E090A3D7-8968-4926-9F35-EF4FB270876D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="276" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="95">
   <si>
     <t>Database No.</t>
   </si>
@@ -2897,7 +2897,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3518C62A-2ABA-4532-ADB0-E26CA60F7C0C}">
-  <dimension ref="A1:P1"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:16">
@@ -2936,6 +2936,178 @@
       </c>
       <c r="P1" t="s">
         <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16">
+      <c r="A2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16">
+      <c r="A3">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16">
+      <c r="A4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16">
+      <c r="A5">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6">
+        <v>61</v>
+      </c>
+      <c r="E6">
+        <v>167</v>
+      </c>
+      <c r="G6">
+        <v>2</v>
+      </c>
+      <c r="H6">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>42</v>
+      </c>
+      <c r="C7" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7">
+        <v>71.8</v>
+      </c>
+      <c r="E7">
+        <v>174</v>
+      </c>
+      <c r="G7">
+        <v>2</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8">
+        <v>100.5</v>
+      </c>
+      <c r="E8">
+        <v>182</v>
+      </c>
+      <c r="G8">
+        <v>2</v>
+      </c>
+      <c r="H8">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>83</v>
+      </c>
+      <c r="D9">
+        <v>60.7</v>
+      </c>
+      <c r="E9">
+        <v>165</v>
+      </c>
+      <c r="G9">
+        <v>2</v>
+      </c>
+      <c r="H9">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16">
+      <c r="A10">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16">
+      <c r="A11">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16">
+      <c r="A12">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16">
+      <c r="A14">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16">
+      <c r="A15">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16">
+      <c r="A16">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1">
+      <c r="A20">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1">
+      <c r="A21">
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add DB5 retargeted files and results
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/shahzaibali/Desktop/TeamProject/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDEB6682-670E-1D46-BC25-19AC66065210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3A1DD3-767B-A546-8683-3A7E1AF4D8CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="34200" windowHeight="21380" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="20140" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
     <sheet name="DB1" sheetId="2" r:id="rId2"/>
     <sheet name="DB2" sheetId="3" r:id="rId3"/>
     <sheet name="DB3" sheetId="4" r:id="rId4"/>
-    <sheet name="DB4" sheetId="5" r:id="rId5"/>
+    <sheet name="DB5" sheetId="5" r:id="rId5"/>
     <sheet name="DB Grouvel" sheetId="6" r:id="rId6"/>
     <sheet name="DB Han" sheetId="7" r:id="rId7"/>
   </sheets>

</xml_diff>

<commit_message>
DB4 & DB5 DB inventory update
</commit_message>
<xml_diff>
--- a/data/database_inventory.xlsx
+++ b/data/database_inventory.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\perla\Documents\AT\TeamProject\GitHub\TeamProject\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rosesharifi/Documents/GitHub/TeamProject/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7EF1EE6-401A-4E3E-AF97-F321F71DE426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A9A62A1-EA7A-7A41-83EC-643873FE09D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="48700" yWindow="-3260" windowWidth="18980" windowHeight="20780" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Main" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="105">
   <si>
     <t>Database No.</t>
   </si>
@@ -383,6 +383,27 @@
   </si>
   <si>
     <t>Walk trials (files)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No ID (Force Status): T06, T10, T12, T22 </t>
+  </si>
+  <si>
+    <t>No ID (Force Status): T04, T10</t>
+  </si>
+  <si>
+    <t>No ID (Force Status) at all</t>
+  </si>
+  <si>
+    <t>No ID (force status): T08, T35, T38</t>
+  </si>
+  <si>
+    <t>No ID at all</t>
+  </si>
+  <si>
+    <t>No ID (force status): T19, T24, T32, T39, T40, T41</t>
+  </si>
+  <si>
+    <t>No ID (force status): T02, T25, T26, T33, T45, T46, T47</t>
   </si>
 </sst>
 </file>
@@ -789,28 +810,28 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R13"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="11.77734375" customWidth="1"/>
-    <col min="2" max="2" width="12.44140625" style="1" customWidth="1"/>
-    <col min="3" max="3" width="18.109375" customWidth="1"/>
-    <col min="4" max="4" width="33.77734375" customWidth="1"/>
+    <col min="1" max="1" width="11.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.5" style="1" customWidth="1"/>
+    <col min="3" max="3" width="18.1640625" customWidth="1"/>
+    <col min="4" max="4" width="33.83203125" customWidth="1"/>
     <col min="5" max="5" width="36" customWidth="1"/>
     <col min="6" max="6" width="23.6640625" style="1" customWidth="1"/>
-    <col min="7" max="7" width="13.44140625" customWidth="1"/>
-    <col min="9" max="9" width="9.77734375" customWidth="1"/>
+    <col min="7" max="7" width="13.5" customWidth="1"/>
+    <col min="9" max="9" width="9.83203125" customWidth="1"/>
     <col min="10" max="10" width="12.6640625" customWidth="1"/>
     <col min="11" max="11" width="14.33203125" customWidth="1"/>
     <col min="12" max="12" width="12.6640625" customWidth="1"/>
     <col min="13" max="13" width="20" customWidth="1"/>
-    <col min="14" max="14" width="28.44140625" customWidth="1"/>
-    <col min="15" max="15" width="24.44140625" customWidth="1"/>
+    <col min="14" max="14" width="28.5" customWidth="1"/>
+    <col min="15" max="15" width="24.5" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
-    <col min="17" max="17" width="40.77734375" style="1" customWidth="1"/>
-    <col min="18" max="18" width="29.77734375" customWidth="1"/>
+    <col min="17" max="17" width="40.83203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="29.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="2" customFormat="1" ht="15.6">
+    <row r="1" spans="1:18" s="2" customFormat="1" ht="17">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -863,7 +884,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="72">
+    <row r="2" spans="1:18" ht="80">
       <c r="A2">
         <v>1</v>
       </c>
@@ -916,7 +937,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="43.2">
+    <row r="3" spans="1:18" ht="48">
       <c r="A3">
         <v>2</v>
       </c>
@@ -960,7 +981,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="4" spans="1:18">
+    <row r="4" spans="1:18" ht="16">
       <c r="A4" s="5">
         <v>3</v>
       </c>
@@ -989,7 +1010,7 @@
       <c r="I8" s="1"/>
       <c r="R8" s="1"/>
     </row>
-    <row r="9" spans="1:18" ht="57.6">
+    <row r="9" spans="1:18" ht="48">
       <c r="B9" s="1" t="s">
         <v>37</v>
       </c>
@@ -1018,7 +1039,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="43.2">
+    <row r="10" spans="1:18" ht="48">
       <c r="B10" s="1" t="s">
         <v>42</v>
       </c>
@@ -1085,7 +1106,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="46.8">
+    <row r="12" spans="1:18" ht="51">
       <c r="B12" s="1" t="s">
         <v>55</v>
       </c>
@@ -1126,7 +1147,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="43.2">
+    <row r="13" spans="1:18" ht="48">
       <c r="B13" s="1" t="s">
         <v>63</v>
       </c>
@@ -1189,18 +1210,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P52"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.109375" customWidth="1"/>
-    <col min="2" max="2" width="10.77734375" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" customWidth="1"/>
+    <col min="1" max="1" width="10.1640625" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.5" customWidth="1"/>
     <col min="4" max="4" width="12.6640625" customWidth="1"/>
     <col min="5" max="5" width="12" customWidth="1"/>
     <col min="6" max="6" width="5.33203125" customWidth="1"/>
-    <col min="7" max="7" width="11.77734375" customWidth="1"/>
+    <col min="7" max="7" width="11.83203125" customWidth="1"/>
     <col min="8" max="8" width="16.6640625" customWidth="1"/>
     <col min="9" max="9" width="17" customWidth="1"/>
-    <col min="10" max="10" width="16.77734375" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
     <col min="11" max="11" width="13" customWidth="1"/>
     <col min="12" max="12" width="9.33203125" customWidth="1"/>
     <col min="16" max="16" width="16.6640625" customWidth="1"/>
@@ -1244,7 +1265,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:16" ht="16">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1276,7 +1297,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:16" ht="16">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1308,7 +1329,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:16" ht="16">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1340,7 +1361,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:16" ht="16">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1372,7 +1393,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:16" ht="16">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1404,7 +1425,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:16" ht="16">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1436,7 +1457,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:16" ht="16">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1468,7 +1489,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:16" ht="16">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1500,7 +1521,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:16" ht="16">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1532,7 +1553,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:16" ht="16">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1564,7 +1585,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:16" ht="16">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1590,7 +1611,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:16" ht="16">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1616,7 +1637,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:16" ht="16">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1642,7 +1663,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:16" ht="16">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1668,7 +1689,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:16" ht="16">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1694,7 +1715,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:16">
+    <row r="17" spans="1:16" ht="16">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1720,7 +1741,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="18" spans="1:16">
+    <row r="18" spans="1:16" ht="16">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1746,7 +1767,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:16">
+    <row r="19" spans="1:16" ht="16">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1772,7 +1793,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="20" spans="1:16">
+    <row r="20" spans="1:16" ht="16">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1798,7 +1819,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:16">
+    <row r="21" spans="1:16" ht="16">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1824,7 +1845,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:16">
+    <row r="22" spans="1:16" ht="16">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1850,7 +1871,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:16">
+    <row r="23" spans="1:16" ht="16">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1876,7 +1897,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="24" spans="1:16">
+    <row r="24" spans="1:16" ht="16">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1902,7 +1923,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:16">
+    <row r="25" spans="1:16" ht="16">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1928,7 +1949,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:16">
+    <row r="26" spans="1:16" ht="16">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1954,7 +1975,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:16">
+    <row r="27" spans="1:16" ht="16">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1980,7 +2001,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:16">
+    <row r="28" spans="1:16" ht="16">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2006,7 +2027,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:16">
+    <row r="29" spans="1:16" ht="16">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2032,7 +2053,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:16">
+    <row r="30" spans="1:16" ht="16">
       <c r="A30">
         <v>29</v>
       </c>
@@ -2058,7 +2079,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:16">
+    <row r="31" spans="1:16" ht="16">
       <c r="A31">
         <v>30</v>
       </c>
@@ -2084,7 +2105,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="32" spans="1:16">
+    <row r="32" spans="1:16" ht="16">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2110,7 +2131,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:16">
+    <row r="33" spans="1:16" ht="16">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2136,7 +2157,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="34" spans="1:16">
+    <row r="34" spans="1:16" ht="16">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2162,7 +2183,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:16">
+    <row r="35" spans="1:16" ht="16">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2188,7 +2209,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="36" spans="1:16">
+    <row r="36" spans="1:16" ht="16">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2214,7 +2235,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
+    <row r="37" spans="1:16" ht="16">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2240,7 +2261,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
+    <row r="38" spans="1:16" ht="16">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2266,7 +2287,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
+    <row r="39" spans="1:16" ht="16">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2292,7 +2313,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="40" spans="1:16">
+    <row r="40" spans="1:16" ht="16">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2318,7 +2339,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:16">
+    <row r="41" spans="1:16" ht="16">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2344,7 +2365,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="42" spans="1:16">
+    <row r="42" spans="1:16" ht="16">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2370,7 +2391,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="43" spans="1:16">
+    <row r="43" spans="1:16" ht="16">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2396,7 +2417,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="44" spans="1:16">
+    <row r="44" spans="1:16" ht="16">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2422,7 +2443,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="45" spans="1:16">
+    <row r="45" spans="1:16" ht="16">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2448,7 +2469,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="46" spans="1:16">
+    <row r="46" spans="1:16" ht="16">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2474,7 +2495,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="47" spans="1:16">
+    <row r="47" spans="1:16" ht="16">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2500,7 +2521,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="48" spans="1:16">
+    <row r="48" spans="1:16" ht="16">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2526,7 +2547,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:16">
+    <row r="49" spans="1:16" ht="16">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2552,7 +2573,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="50" spans="1:16">
+    <row r="50" spans="1:16" ht="16">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2578,7 +2599,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="51" spans="1:16">
+    <row r="51" spans="1:16" ht="16">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2619,14 +2640,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L15"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="10.44140625" customWidth="1"/>
+    <col min="8" max="8" width="10.5" customWidth="1"/>
     <col min="9" max="9" width="30.6640625" customWidth="1"/>
-    <col min="10" max="10" width="33.109375" customWidth="1"/>
+    <col min="10" max="10" width="33.1640625" customWidth="1"/>
     <col min="11" max="11" width="36.6640625" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" customWidth="1"/>
-    <col min="14" max="14" width="14.109375" customWidth="1"/>
+    <col min="12" max="12" width="15.5" customWidth="1"/>
+    <col min="14" max="14" width="14.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -3005,7 +3026,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:P21"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:16">
       <c r="A1" t="s">
@@ -3298,9 +3319,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D22FEE7-983F-4E6D-B518-6357D6EFC8AC}">
   <dimension ref="A1:P58"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="46.33203125" customWidth="1"/>
+    <col min="6" max="6" width="0.83203125" customWidth="1"/>
+    <col min="7" max="7" width="6.6640625" customWidth="1"/>
+    <col min="8" max="8" width="7.1640625" customWidth="1"/>
+    <col min="9" max="9" width="30.83203125" customWidth="1"/>
+    <col min="10" max="10" width="48.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -3649,7 +3674,9 @@
       <c r="H14" s="11">
         <v>22</v>
       </c>
-      <c r="I14" s="11"/>
+      <c r="I14" s="11" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="15" spans="1:16">
       <c r="A15">
@@ -3724,7 +3751,9 @@
       <c r="H17" s="11">
         <v>21</v>
       </c>
-      <c r="I17" s="11"/>
+      <c r="I17" s="11" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18">
@@ -3774,7 +3803,9 @@
       <c r="H19" s="11">
         <v>21</v>
       </c>
-      <c r="I19" s="11"/>
+      <c r="I19" s="11" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20">
@@ -4277,12 +4308,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:P52"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="9.77734375" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375"/>
+    <col min="1" max="1" width="9.83203125" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125"/>
     <col min="4" max="4" width="13.6640625" customWidth="1"/>
-    <col min="5" max="5" width="12.44140625" customWidth="1"/>
+    <col min="5" max="5" width="12.5" customWidth="1"/>
+    <col min="8" max="8" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:16">
@@ -4578,7 +4610,7 @@
         <v>166.7</v>
       </c>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:8">
       <c r="A17">
         <v>16</v>
       </c>
@@ -4595,7 +4627,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:8">
       <c r="A18">
         <v>17</v>
       </c>
@@ -4612,7 +4644,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:8">
       <c r="A19">
         <v>18</v>
       </c>
@@ -4629,7 +4661,7 @@
         <v>173.7</v>
       </c>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:8">
       <c r="A20">
         <v>19</v>
       </c>
@@ -4646,7 +4678,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:8">
       <c r="A21">
         <v>20</v>
       </c>
@@ -4663,7 +4695,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:8">
       <c r="A22">
         <v>21</v>
       </c>
@@ -4680,7 +4712,7 @@
         <v>172.5</v>
       </c>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:8">
       <c r="A23">
         <v>22</v>
       </c>
@@ -4697,7 +4729,7 @@
         <v>184.5</v>
       </c>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:8">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4714,7 +4746,7 @@
         <v>172.5</v>
       </c>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:8">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4731,7 +4763,7 @@
         <v>173.5</v>
       </c>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:8">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4748,7 +4780,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="27" spans="1:5">
+    <row r="27" spans="1:8">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4765,7 +4797,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="28" spans="1:5">
+    <row r="28" spans="1:8">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4782,7 +4814,7 @@
         <v>166.2</v>
       </c>
     </row>
-    <row r="29" spans="1:5">
+    <row r="29" spans="1:8">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4799,7 +4831,7 @@
         <v>172.5</v>
       </c>
     </row>
-    <row r="30" spans="1:5">
+    <row r="30" spans="1:8">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4816,7 +4848,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="31" spans="1:5">
+    <row r="31" spans="1:8">
       <c r="A31">
         <v>30</v>
       </c>
@@ -4833,7 +4865,7 @@
         <v>174.5</v>
       </c>
     </row>
-    <row r="32" spans="1:5">
+    <row r="32" spans="1:8">
       <c r="A32">
         <v>31</v>
       </c>
@@ -4849,8 +4881,11 @@
       <c r="E32">
         <v>183</v>
       </c>
-    </row>
-    <row r="33" spans="1:5">
+      <c r="H32" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
       <c r="A33">
         <v>32</v>
       </c>
@@ -4866,8 +4901,11 @@
       <c r="E33">
         <v>169</v>
       </c>
-    </row>
-    <row r="34" spans="1:5">
+      <c r="H33" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
       <c r="A34">
         <v>33</v>
       </c>
@@ -4883,8 +4921,11 @@
       <c r="E34">
         <v>161</v>
       </c>
-    </row>
-    <row r="35" spans="1:5">
+      <c r="H34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35">
         <v>34</v>
       </c>
@@ -4900,8 +4941,11 @@
       <c r="E35">
         <v>171.5</v>
       </c>
-    </row>
-    <row r="36" spans="1:5">
+      <c r="H35" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
       <c r="A36">
         <v>35</v>
       </c>
@@ -4917,8 +4961,11 @@
       <c r="E36">
         <v>175.5</v>
       </c>
-    </row>
-    <row r="37" spans="1:5">
+      <c r="H36" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4934,8 +4981,11 @@
       <c r="E37">
         <v>169.6</v>
       </c>
-    </row>
-    <row r="38" spans="1:5">
+      <c r="H37" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
       <c r="A38">
         <v>37</v>
       </c>
@@ -4951,8 +5001,11 @@
       <c r="E38">
         <v>186.6</v>
       </c>
-    </row>
-    <row r="39" spans="1:5">
+      <c r="H38" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
       <c r="A39">
         <v>38</v>
       </c>
@@ -4968,8 +5021,11 @@
       <c r="E39">
         <v>180.7</v>
       </c>
-    </row>
-    <row r="40" spans="1:5">
+      <c r="H39" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4985,8 +5041,11 @@
       <c r="E40">
         <v>170</v>
       </c>
-    </row>
-    <row r="41" spans="1:5">
+      <c r="H40" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41">
         <v>40</v>
       </c>
@@ -5002,8 +5061,11 @@
       <c r="E41">
         <v>183.6</v>
       </c>
-    </row>
-    <row r="42" spans="1:5">
+      <c r="H41" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42">
         <v>41</v>
       </c>
@@ -5020,7 +5082,7 @@
         <v>185.5</v>
       </c>
     </row>
-    <row r="43" spans="1:5">
+    <row r="43" spans="1:8">
       <c r="A43">
         <v>42</v>
       </c>
@@ -5037,7 +5099,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="44" spans="1:5">
+    <row r="44" spans="1:8">
       <c r="A44">
         <v>43</v>
       </c>
@@ -5054,7 +5116,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="45" spans="1:5">
+    <row r="45" spans="1:8">
       <c r="A45">
         <v>44</v>
       </c>
@@ -5071,7 +5133,7 @@
         <v>164.5</v>
       </c>
     </row>
-    <row r="46" spans="1:5">
+    <row r="46" spans="1:8">
       <c r="A46">
         <v>45</v>
       </c>
@@ -5088,7 +5150,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="47" spans="1:5">
+    <row r="47" spans="1:8">
       <c r="A47">
         <v>46</v>
       </c>
@@ -5105,7 +5167,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="48" spans="1:5">
+    <row r="48" spans="1:8">
       <c r="A48">
         <v>47</v>
       </c>
@@ -5199,13 +5261,13 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L13"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="10.77734375" customWidth="1"/>
-    <col min="9" max="9" width="28.77734375" customWidth="1"/>
-    <col min="10" max="10" width="33.109375" customWidth="1"/>
+    <col min="8" max="8" width="10.83203125" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+    <col min="10" max="10" width="33.1640625" customWidth="1"/>
     <col min="11" max="11" width="36.6640625" customWidth="1"/>
-    <col min="12" max="12" width="13.44140625" customWidth="1"/>
+    <col min="12" max="12" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -5497,12 +5559,12 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col min="8" max="8" width="11.44140625" customWidth="1"/>
-    <col min="9" max="9" width="29.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.5" customWidth="1"/>
+    <col min="9" max="9" width="29.83203125" customWidth="1"/>
     <col min="10" max="10" width="34" customWidth="1"/>
-    <col min="11" max="11" width="36.77734375" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
     <col min="12" max="12" width="13" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>